<commit_message>
Agregar pestañas Acopios y Certificados, reemplazar Excel actualizado
- Nuevos endpoints /api/acopios y /api/certificados que parsean las hojas
  Acopios, Básico $, Básico USD Plaza y Básico USD CIF (sin hardcodear
  valores, todo sale del Excel real).
- Pestaña General ahora incluye la evolución del Ajuste Paramétrico
  (hoja AP, columnas AL/AM).
- Dashboard.jsx replica el layout de 3 pestañas (General/Acopios/
  Certificados) del prototipo v5, con selector de moneda e IVA en
  Certificados.
- Reemplazado data/detalle_pagos_CEAOSA.xlsx por la versión actualizada.
- Validado contra el brief: consolidado en USD con TC=39.5 coincide
  exactamente con D124/E124/F124/I146/I147 de la hoja Resumen; totales
  de las 3 hojas de certificados e IVA coinciden con las celdas reales.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/detalle_pagos_CEAOSA.xlsx
+++ b/data/detalle_pagos_CEAOSA.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ddcuru-my.sharepoint.com/personal/acarrasco_ddc_com_uy/Documents/DDC Obra/06_LIV District/02_Rubrados y Memorias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5469" documentId="8_{E6E6E29B-3EF0-4132-A1BA-B0532C1168ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{683605E2-B961-4C38-93F1-FE77664E3F1D}"/>
+  <xr:revisionPtr revIDLastSave="5510" documentId="8_{E6E6E29B-3EF0-4132-A1BA-B0532C1168ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{56CF6D2B-1717-44B4-806E-E971E5223203}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="819" xr2:uid="{67942048-5DB5-4941-BA24-94B26BD83A64}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="819" activeTab="9" xr2:uid="{67942048-5DB5-4941-BA24-94B26BD83A64}"/>
   </bookViews>
   <sheets>
     <sheet name="Resumen" sheetId="11" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="879" uniqueCount="344">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="881" uniqueCount="345">
   <si>
     <t>N° Certificado</t>
   </si>
@@ -1022,9 +1022,6 @@
     <t>A-5528</t>
   </si>
   <si>
-    <t>A-5545</t>
-  </si>
-  <si>
     <t>Avance básico USD CIF</t>
   </si>
   <si>
@@ -1086,6 +1083,12 @@
   </si>
   <si>
     <t xml:space="preserve">tc </t>
+  </si>
+  <si>
+    <t>A-5545 (A-1964)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se descuenta de AP básico </t>
   </si>
 </sst>
 </file>
@@ -1398,7 +1401,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="229">
+  <cellXfs count="230">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1656,9 +1659,6 @@
     <xf numFmtId="14" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1687,38 +1687,8 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="2" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="2" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1816,9 +1786,6 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="17" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1867,6 +1834,9 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="14" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -1906,6 +1876,36 @@
     <xf numFmtId="17" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="10" fontId="0" fillId="2" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="2" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="17" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -1920,6 +1920,12 @@
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -31264,15 +31270,15 @@
     </row>
     <row r="4" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B4" s="112"/>
-      <c r="C4" s="169" t="s">
+      <c r="C4" s="158" t="s">
         <v>253</v>
       </c>
-      <c r="D4" s="169"/>
-      <c r="H4" s="170" t="s">
+      <c r="D4" s="158"/>
+      <c r="H4" s="159" t="s">
         <v>254</v>
       </c>
-      <c r="I4" s="171"/>
-      <c r="J4" s="172"/>
+      <c r="I4" s="160"/>
+      <c r="J4" s="161"/>
       <c r="K4" s="113"/>
     </row>
     <row r="5" spans="2:16" x14ac:dyDescent="0.25">
@@ -31358,17 +31364,17 @@
     </row>
     <row r="10" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B10" s="112"/>
-      <c r="C10" s="169" t="s">
+      <c r="C10" s="158" t="s">
         <v>257</v>
       </c>
-      <c r="D10" s="169"/>
-      <c r="E10" s="169"/>
-      <c r="F10" s="169"/>
+      <c r="D10" s="158"/>
+      <c r="E10" s="158"/>
+      <c r="F10" s="158"/>
       <c r="K10" s="113"/>
     </row>
     <row r="11" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B11" s="112"/>
-      <c r="C11" s="168" t="s">
+      <c r="C11" s="157" t="s">
         <v>254</v>
       </c>
       <c r="D11" s="2" t="s">
@@ -31381,16 +31387,16 @@
         <f>+E11*D5</f>
         <v>8935691.8000000007</v>
       </c>
-      <c r="H11" s="170" t="s">
+      <c r="H11" s="159" t="s">
         <v>255</v>
       </c>
-      <c r="I11" s="171"/>
-      <c r="J11" s="172"/>
+      <c r="I11" s="160"/>
+      <c r="J11" s="161"/>
       <c r="K11" s="113"/>
     </row>
     <row r="12" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B12" s="112"/>
-      <c r="C12" s="168"/>
+      <c r="C12" s="157"/>
       <c r="D12" s="2" t="s">
         <v>10</v>
       </c>
@@ -31405,7 +31411,7 @@
     </row>
     <row r="13" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B13" s="112"/>
-      <c r="C13" s="168"/>
+      <c r="C13" s="157"/>
       <c r="D13" s="2" t="s">
         <v>11</v>
       </c>
@@ -31429,10 +31435,10 @@
     </row>
     <row r="14" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B14" s="112"/>
-      <c r="C14" s="161" t="s">
+      <c r="C14" s="150" t="s">
         <v>5</v>
       </c>
-      <c r="D14" s="162"/>
+      <c r="D14" s="151"/>
       <c r="E14" s="98">
         <f>+SUM(E11:E13)</f>
         <v>0.05</v>
@@ -31455,7 +31461,7 @@
     </row>
     <row r="15" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B15" s="112"/>
-      <c r="C15" s="168" t="s">
+      <c r="C15" s="157" t="s">
         <v>255</v>
       </c>
       <c r="D15" s="2" t="s">
@@ -31482,7 +31488,7 @@
     </row>
     <row r="16" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B16" s="112"/>
-      <c r="C16" s="168"/>
+      <c r="C16" s="157"/>
       <c r="D16" s="2" t="s">
         <v>10</v>
       </c>
@@ -31507,7 +31513,7 @@
     </row>
     <row r="17" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B17" s="112"/>
-      <c r="C17" s="168"/>
+      <c r="C17" s="157"/>
       <c r="D17" s="2" t="s">
         <v>11</v>
       </c>
@@ -31522,10 +31528,10 @@
     </row>
     <row r="18" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B18" s="112"/>
-      <c r="C18" s="161" t="s">
+      <c r="C18" s="150" t="s">
         <v>5</v>
       </c>
-      <c r="D18" s="162"/>
+      <c r="D18" s="151"/>
       <c r="E18" s="98">
         <f>+SUM(E15:E17)</f>
         <v>0.05</v>
@@ -31534,16 +31540,16 @@
         <f>+SUM(F15:F17)</f>
         <v>656526.14000000013</v>
       </c>
-      <c r="H18" s="170" t="s">
+      <c r="H18" s="159" t="s">
         <v>256</v>
       </c>
-      <c r="I18" s="171"/>
-      <c r="J18" s="172"/>
+      <c r="I18" s="160"/>
+      <c r="J18" s="161"/>
       <c r="K18" s="113"/>
     </row>
     <row r="19" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B19" s="112"/>
-      <c r="C19" s="168" t="s">
+      <c r="C19" s="157" t="s">
         <v>256</v>
       </c>
       <c r="D19" s="2" t="s">
@@ -31560,7 +31566,7 @@
     </row>
     <row r="20" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B20" s="112"/>
-      <c r="C20" s="168"/>
+      <c r="C20" s="157"/>
       <c r="D20" s="2" t="s">
         <v>10</v>
       </c>
@@ -31584,7 +31590,7 @@
     </row>
     <row r="21" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B21" s="112"/>
-      <c r="C21" s="168"/>
+      <c r="C21" s="157"/>
       <c r="D21" s="2" t="s">
         <v>11</v>
       </c>
@@ -31609,10 +31615,10 @@
     </row>
     <row r="22" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B22" s="112"/>
-      <c r="C22" s="161" t="s">
+      <c r="C22" s="150" t="s">
         <v>5</v>
       </c>
-      <c r="D22" s="162"/>
+      <c r="D22" s="151"/>
       <c r="E22" s="98">
         <f>+SUM(E19:E21)</f>
         <v>0.05</v>
@@ -31656,11 +31662,11 @@
     </row>
     <row r="25" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B25" s="112"/>
-      <c r="C25" s="163" t="s">
+      <c r="C25" s="152" t="s">
         <v>258</v>
       </c>
-      <c r="D25" s="164"/>
-      <c r="E25" s="165"/>
+      <c r="D25" s="153"/>
+      <c r="E25" s="154"/>
       <c r="K25" s="113"/>
     </row>
     <row r="26" spans="2:11" x14ac:dyDescent="0.25">
@@ -31668,7 +31674,7 @@
       <c r="C26" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="D26" s="166">
+      <c r="D26" s="155">
         <v>0.05</v>
       </c>
       <c r="E26" s="27">
@@ -31682,7 +31688,7 @@
       <c r="C27" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="D27" s="166"/>
+      <c r="D27" s="155"/>
       <c r="E27" s="27">
         <f>+$D$26*D6</f>
         <v>31870.2</v>
@@ -31694,7 +31700,7 @@
       <c r="C28" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="D28" s="166"/>
+      <c r="D28" s="155"/>
       <c r="E28" s="27">
         <f>+$D$26*D7</f>
         <v>22565.15</v>
@@ -31711,11 +31717,11 @@
     </row>
     <row r="31" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B31" s="112"/>
-      <c r="C31" s="163" t="s">
+      <c r="C31" s="152" t="s">
         <v>250</v>
       </c>
-      <c r="D31" s="164"/>
-      <c r="E31" s="165"/>
+      <c r="D31" s="153"/>
+      <c r="E31" s="154"/>
       <c r="K31" s="113"/>
     </row>
     <row r="32" spans="2:11" x14ac:dyDescent="0.25">
@@ -31723,7 +31729,7 @@
       <c r="C32" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="D32" s="173">
+      <c r="D32" s="162">
         <v>2.5000000000000001E-2</v>
       </c>
       <c r="E32" s="27">
@@ -31737,7 +31743,7 @@
       <c r="C33" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="D33" s="173"/>
+      <c r="D33" s="162"/>
       <c r="E33" s="27">
         <f>+$D$32*D6</f>
         <v>15935.1</v>
@@ -31749,7 +31755,7 @@
       <c r="C34" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="D34" s="173"/>
+      <c r="D34" s="162"/>
       <c r="E34" s="27">
         <f>+$D$32*D7</f>
         <v>11282.575000000001</v>
@@ -31796,15 +31802,15 @@
     </row>
     <row r="40" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B40" s="112"/>
-      <c r="C40" s="169" t="s">
+      <c r="C40" s="158" t="s">
         <v>253</v>
       </c>
-      <c r="D40" s="169"/>
-      <c r="H40" s="170" t="s">
+      <c r="D40" s="158"/>
+      <c r="H40" s="159" t="s">
         <v>254</v>
       </c>
-      <c r="I40" s="171"/>
-      <c r="J40" s="172"/>
+      <c r="I40" s="160"/>
+      <c r="J40" s="161"/>
       <c r="K40" s="113"/>
     </row>
     <row r="41" spans="2:11" x14ac:dyDescent="0.25">
@@ -31892,17 +31898,17 @@
     </row>
     <row r="46" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B46" s="112"/>
-      <c r="C46" s="169" t="s">
+      <c r="C46" s="158" t="s">
         <v>257</v>
       </c>
-      <c r="D46" s="169"/>
-      <c r="E46" s="169"/>
-      <c r="F46" s="169"/>
+      <c r="D46" s="158"/>
+      <c r="E46" s="158"/>
+      <c r="F46" s="158"/>
       <c r="K46" s="113"/>
     </row>
     <row r="47" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B47" s="112"/>
-      <c r="C47" s="168" t="s">
+      <c r="C47" s="157" t="s">
         <v>254</v>
       </c>
       <c r="D47" s="2" t="s">
@@ -31915,16 +31921,16 @@
         <f>+E47*D41</f>
         <v>226220.04556962024</v>
       </c>
-      <c r="H47" s="170" t="s">
+      <c r="H47" s="159" t="s">
         <v>255</v>
       </c>
-      <c r="I47" s="171"/>
-      <c r="J47" s="172"/>
+      <c r="I47" s="160"/>
+      <c r="J47" s="161"/>
       <c r="K47" s="113"/>
     </row>
     <row r="48" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B48" s="112"/>
-      <c r="C48" s="168"/>
+      <c r="C48" s="157"/>
       <c r="D48" s="2" t="s">
         <v>10</v>
       </c>
@@ -31939,7 +31945,7 @@
     </row>
     <row r="49" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B49" s="112"/>
-      <c r="C49" s="168"/>
+      <c r="C49" s="157"/>
       <c r="D49" s="2" t="s">
         <v>11</v>
       </c>
@@ -31963,10 +31969,10 @@
     </row>
     <row r="50" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B50" s="112"/>
-      <c r="C50" s="161" t="s">
+      <c r="C50" s="150" t="s">
         <v>5</v>
       </c>
-      <c r="D50" s="162"/>
+      <c r="D50" s="151"/>
       <c r="E50" s="98">
         <f>+SUM(E47:E49)</f>
         <v>0.05</v>
@@ -31989,7 +31995,7 @@
     </row>
     <row r="51" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B51" s="112"/>
-      <c r="C51" s="168" t="s">
+      <c r="C51" s="157" t="s">
         <v>255</v>
       </c>
       <c r="D51" s="2" t="s">
@@ -32016,7 +32022,7 @@
     </row>
     <row r="52" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B52" s="112"/>
-      <c r="C52" s="168"/>
+      <c r="C52" s="157"/>
       <c r="D52" s="2" t="s">
         <v>10</v>
       </c>
@@ -32041,7 +32047,7 @@
     </row>
     <row r="53" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B53" s="112"/>
-      <c r="C53" s="168"/>
+      <c r="C53" s="157"/>
       <c r="D53" s="2" t="s">
         <v>11</v>
       </c>
@@ -32056,10 +32062,10 @@
     </row>
     <row r="54" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B54" s="112"/>
-      <c r="C54" s="161" t="s">
+      <c r="C54" s="150" t="s">
         <v>5</v>
       </c>
-      <c r="D54" s="162"/>
+      <c r="D54" s="151"/>
       <c r="E54" s="98">
         <f>+SUM(E51:E53)</f>
         <v>0.05</v>
@@ -32068,16 +32074,16 @@
         <f>+SUM(F51:F53)</f>
         <v>656526.14000000013</v>
       </c>
-      <c r="H54" s="170" t="s">
+      <c r="H54" s="159" t="s">
         <v>256</v>
       </c>
-      <c r="I54" s="171"/>
-      <c r="J54" s="172"/>
+      <c r="I54" s="160"/>
+      <c r="J54" s="161"/>
       <c r="K54" s="113"/>
     </row>
     <row r="55" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B55" s="112"/>
-      <c r="C55" s="168" t="s">
+      <c r="C55" s="157" t="s">
         <v>256</v>
       </c>
       <c r="D55" s="2" t="s">
@@ -32094,7 +32100,7 @@
     </row>
     <row r="56" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B56" s="112"/>
-      <c r="C56" s="168"/>
+      <c r="C56" s="157"/>
       <c r="D56" s="2" t="s">
         <v>10</v>
       </c>
@@ -32118,7 +32124,7 @@
     </row>
     <row r="57" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B57" s="112"/>
-      <c r="C57" s="168"/>
+      <c r="C57" s="157"/>
       <c r="D57" s="2" t="s">
         <v>11</v>
       </c>
@@ -32143,10 +32149,10 @@
     </row>
     <row r="58" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B58" s="112"/>
-      <c r="C58" s="161" t="s">
+      <c r="C58" s="150" t="s">
         <v>5</v>
       </c>
-      <c r="D58" s="162"/>
+      <c r="D58" s="151"/>
       <c r="E58" s="98">
         <f>+SUM(E55:E57)</f>
         <v>0.05</v>
@@ -32193,11 +32199,11 @@
     </row>
     <row r="61" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B61" s="112"/>
-      <c r="C61" s="163" t="s">
+      <c r="C61" s="152" t="s">
         <v>258</v>
       </c>
-      <c r="D61" s="164"/>
-      <c r="E61" s="165"/>
+      <c r="D61" s="153"/>
+      <c r="E61" s="154"/>
       <c r="K61" s="113"/>
     </row>
     <row r="62" spans="2:11" x14ac:dyDescent="0.25">
@@ -32205,7 +32211,7 @@
       <c r="C62" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="D62" s="166">
+      <c r="D62" s="155">
         <v>0.05</v>
       </c>
       <c r="E62" s="27">
@@ -32219,7 +32225,7 @@
       <c r="C63" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="D63" s="166"/>
+      <c r="D63" s="155"/>
       <c r="E63" s="27">
         <f>+$D$26*D42</f>
         <v>31870.2</v>
@@ -32231,7 +32237,7 @@
       <c r="C64" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="D64" s="166"/>
+      <c r="D64" s="155"/>
       <c r="E64" s="27">
         <f>+$D$26*D43</f>
         <v>22565.15</v>
@@ -32248,11 +32254,11 @@
     </row>
     <row r="67" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B67" s="112"/>
-      <c r="C67" s="163" t="s">
+      <c r="C67" s="152" t="s">
         <v>250</v>
       </c>
-      <c r="D67" s="164"/>
-      <c r="E67" s="165"/>
+      <c r="D67" s="153"/>
+      <c r="E67" s="154"/>
       <c r="K67" s="113"/>
     </row>
     <row r="68" spans="2:11" x14ac:dyDescent="0.25">
@@ -32260,7 +32266,7 @@
       <c r="C68" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="D68" s="173">
+      <c r="D68" s="162">
         <v>2.5000000000000001E-2</v>
       </c>
       <c r="E68" s="27">
@@ -32274,7 +32280,7 @@
       <c r="C69" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="D69" s="173"/>
+      <c r="D69" s="162"/>
       <c r="E69" s="27">
         <f>+$D$32*D42</f>
         <v>15935.1</v>
@@ -32286,7 +32292,7 @@
       <c r="C70" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="D70" s="173"/>
+      <c r="D70" s="162"/>
       <c r="E70" s="27">
         <f>+$D$32*D43</f>
         <v>11282.575000000001</v>
@@ -32330,25 +32336,25 @@
     </row>
     <row r="77" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B77" s="112"/>
-      <c r="C77" s="169" t="s">
+      <c r="C77" s="158" t="s">
         <v>271</v>
       </c>
-      <c r="D77" s="169"/>
-      <c r="E77" s="169"/>
-      <c r="F77" s="169"/>
-      <c r="H77" s="170" t="s">
+      <c r="D77" s="158"/>
+      <c r="E77" s="158"/>
+      <c r="F77" s="158"/>
+      <c r="H77" s="159" t="s">
         <v>254</v>
       </c>
-      <c r="I77" s="171"/>
-      <c r="J77" s="172"/>
+      <c r="I77" s="160"/>
+      <c r="J77" s="161"/>
       <c r="K77" s="113"/>
     </row>
     <row r="78" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B78" s="112"/>
-      <c r="C78" s="169" t="s">
+      <c r="C78" s="158" t="s">
         <v>253</v>
       </c>
-      <c r="D78" s="169"/>
+      <c r="D78" s="158"/>
       <c r="E78" s="3" t="s">
         <v>44</v>
       </c>
@@ -32479,12 +32485,12 @@
     </row>
     <row r="84" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B84" s="112"/>
-      <c r="C84" s="169" t="s">
+      <c r="C84" s="158" t="s">
         <v>257</v>
       </c>
-      <c r="D84" s="169"/>
-      <c r="E84" s="169"/>
-      <c r="F84" s="169"/>
+      <c r="D84" s="158"/>
+      <c r="E84" s="158"/>
+      <c r="F84" s="158"/>
       <c r="H84" s="2" t="s">
         <v>306</v>
       </c>
@@ -32500,7 +32506,7 @@
     </row>
     <row r="85" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B85" s="112"/>
-      <c r="C85" s="168" t="s">
+      <c r="C85" s="157" t="s">
         <v>254</v>
       </c>
       <c r="D85" s="2" t="s">
@@ -32528,7 +32534,7 @@
     </row>
     <row r="86" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B86" s="112"/>
-      <c r="C86" s="168"/>
+      <c r="C86" s="157"/>
       <c r="D86" s="2" t="s">
         <v>10</v>
       </c>
@@ -32543,7 +32549,7 @@
     </row>
     <row r="87" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B87" s="112"/>
-      <c r="C87" s="168"/>
+      <c r="C87" s="157"/>
       <c r="D87" s="2" t="s">
         <v>11</v>
       </c>
@@ -32554,19 +32560,19 @@
         <f>+'Básico $'!K25</f>
         <v>1200403.3780732199</v>
       </c>
-      <c r="H87" s="170" t="s">
+      <c r="H87" s="159" t="s">
         <v>255</v>
       </c>
-      <c r="I87" s="171"/>
-      <c r="J87" s="172"/>
+      <c r="I87" s="160"/>
+      <c r="J87" s="161"/>
       <c r="K87" s="113"/>
     </row>
     <row r="88" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B88" s="112"/>
-      <c r="C88" s="161" t="s">
+      <c r="C88" s="150" t="s">
         <v>5</v>
       </c>
-      <c r="D88" s="162"/>
+      <c r="D88" s="151"/>
       <c r="E88" s="98">
         <f>+SUM(E85:E87)</f>
         <v>0.05</v>
@@ -32579,7 +32585,7 @@
     </row>
     <row r="89" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B89" s="112"/>
-      <c r="C89" s="168" t="s">
+      <c r="C89" s="157" t="s">
         <v>255</v>
       </c>
       <c r="D89" s="2" t="s">
@@ -32604,7 +32610,7 @@
     </row>
     <row r="90" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B90" s="112"/>
-      <c r="C90" s="168"/>
+      <c r="C90" s="157"/>
       <c r="D90" s="2" t="s">
         <v>10</v>
       </c>
@@ -32630,7 +32636,7 @@
     </row>
     <row r="91" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B91" s="112"/>
-      <c r="C91" s="168"/>
+      <c r="C91" s="157"/>
       <c r="D91" s="2" t="s">
         <v>11</v>
       </c>
@@ -32656,10 +32662,10 @@
     </row>
     <row r="92" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B92" s="112"/>
-      <c r="C92" s="161" t="s">
+      <c r="C92" s="150" t="s">
         <v>5</v>
       </c>
-      <c r="D92" s="162"/>
+      <c r="D92" s="151"/>
       <c r="E92" s="98">
         <f>+SUM(E89:E91)</f>
         <v>0.05</v>
@@ -32683,7 +32689,7 @@
     </row>
     <row r="93" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B93" s="112"/>
-      <c r="C93" s="168" t="s">
+      <c r="C93" s="157" t="s">
         <v>256</v>
       </c>
       <c r="D93" s="2" t="s">
@@ -32711,7 +32717,7 @@
     </row>
     <row r="94" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B94" s="112"/>
-      <c r="C94" s="168"/>
+      <c r="C94" s="157"/>
       <c r="D94" s="2" t="s">
         <v>10</v>
       </c>
@@ -32737,7 +32743,7 @@
     </row>
     <row r="95" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B95" s="112"/>
-      <c r="C95" s="168"/>
+      <c r="C95" s="157"/>
       <c r="D95" s="2" t="s">
         <v>11</v>
       </c>
@@ -32752,10 +32758,10 @@
     </row>
     <row r="96" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B96" s="112"/>
-      <c r="C96" s="161" t="s">
+      <c r="C96" s="150" t="s">
         <v>5</v>
       </c>
-      <c r="D96" s="162"/>
+      <c r="D96" s="151"/>
       <c r="E96" s="98">
         <f>+SUM(E93:E95)</f>
         <v>0.05</v>
@@ -32764,11 +32770,11 @@
         <f>+F93+F94+F95</f>
         <v>5239.2570000000005</v>
       </c>
-      <c r="H96" s="170" t="s">
+      <c r="H96" s="159" t="s">
         <v>256</v>
       </c>
-      <c r="I96" s="171"/>
-      <c r="J96" s="172"/>
+      <c r="I96" s="160"/>
+      <c r="J96" s="161"/>
       <c r="K96" s="113"/>
     </row>
     <row r="97" spans="2:11" x14ac:dyDescent="0.25">
@@ -32792,11 +32798,11 @@
     </row>
     <row r="99" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B99" s="112"/>
-      <c r="C99" s="163" t="s">
+      <c r="C99" s="152" t="s">
         <v>258</v>
       </c>
-      <c r="D99" s="164"/>
-      <c r="E99" s="165"/>
+      <c r="D99" s="153"/>
+      <c r="E99" s="154"/>
       <c r="H99" s="2" t="s">
         <v>259</v>
       </c>
@@ -32815,7 +32821,7 @@
       <c r="C100" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="D100" s="166">
+      <c r="D100" s="155">
         <v>0.05</v>
       </c>
       <c r="E100" s="27">
@@ -32841,7 +32847,7 @@
       <c r="C101" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="D101" s="166"/>
+      <c r="D101" s="155"/>
       <c r="E101" s="27">
         <f>+'Básico USD Plaza'!W8</f>
         <v>9663.2459999999992</v>
@@ -32865,7 +32871,7 @@
       <c r="C102" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="D102" s="166"/>
+      <c r="D102" s="155"/>
       <c r="E102" s="7">
         <f>+'Básico USD CIF'!W6</f>
         <v>5239.2570000000005</v>
@@ -32889,7 +32895,7 @@
       <c r="C103" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="D103" s="166"/>
+      <c r="D103" s="155"/>
       <c r="E103" s="7">
         <f>+AP!Z6</f>
         <v>702053.87300000014</v>
@@ -32913,7 +32919,7 @@
       <c r="C104" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="D104" s="166"/>
+      <c r="D104" s="155"/>
       <c r="E104" s="7">
         <f>+'AP Adicionales'!V7</f>
         <v>1567.7080000000001</v>
@@ -32925,7 +32931,7 @@
       <c r="C105" s="2" t="s">
         <v>274</v>
       </c>
-      <c r="D105" s="166"/>
+      <c r="D105" s="155"/>
       <c r="E105" s="7">
         <f>+'AyD $'!V6</f>
         <v>22772.803001667893</v>
@@ -32937,7 +32943,7 @@
       <c r="C106" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="D106" s="166"/>
+      <c r="D106" s="155"/>
       <c r="E106" s="7">
         <f>+'AYD USD Plaza '!V7</f>
         <v>5200.5317757272096</v>
@@ -32949,7 +32955,7 @@
       <c r="C107" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="D107" s="166"/>
+      <c r="D107" s="155"/>
       <c r="E107" s="7">
         <f>+'Básico USD CIF'!W6</f>
         <v>5239.2570000000005</v>
@@ -32962,11 +32968,11 @@
     </row>
     <row r="109" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B109" s="112"/>
-      <c r="C109" s="163" t="s">
+      <c r="C109" s="152" t="s">
         <v>250</v>
       </c>
-      <c r="D109" s="164"/>
-      <c r="E109" s="165"/>
+      <c r="D109" s="153"/>
+      <c r="E109" s="154"/>
       <c r="K109" s="113"/>
     </row>
     <row r="110" spans="2:11" x14ac:dyDescent="0.25">
@@ -32974,7 +32980,7 @@
       <c r="C110" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="D110" s="167">
+      <c r="D110" s="156">
         <v>2.5000000000000001E-2</v>
       </c>
       <c r="E110" s="27">
@@ -32988,7 +32994,7 @@
       <c r="C111" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="D111" s="167"/>
+      <c r="D111" s="156"/>
       <c r="E111" s="27">
         <f>+'Básico USD Plaza'!W9</f>
         <v>4831.6229999999996</v>
@@ -33000,7 +33006,7 @@
       <c r="C112" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="D112" s="167"/>
+      <c r="D112" s="156"/>
       <c r="E112" s="27">
         <f>+'Básico USD CIF'!W7</f>
         <v>2619.6285000000003</v>
@@ -33012,7 +33018,7 @@
       <c r="C113" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="D113" s="167"/>
+      <c r="D113" s="156"/>
       <c r="E113" s="27">
         <f>+AP!Z7</f>
         <v>351026.93650000007</v>
@@ -33052,22 +33058,22 @@
     </row>
     <row r="119" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B119" s="112"/>
-      <c r="C119" s="169" t="s">
+      <c r="C119" s="158" t="s">
         <v>281</v>
       </c>
-      <c r="D119" s="169"/>
-      <c r="E119" s="169"/>
-      <c r="F119" s="169"/>
-      <c r="G119" s="169"/>
-      <c r="H119" s="169"/>
+      <c r="D119" s="158"/>
+      <c r="E119" s="158"/>
+      <c r="F119" s="158"/>
+      <c r="G119" s="158"/>
+      <c r="H119" s="158"/>
       <c r="K119" s="113"/>
     </row>
     <row r="120" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B120" s="112"/>
-      <c r="C120" s="169" t="s">
+      <c r="C120" s="158" t="s">
         <v>253</v>
       </c>
-      <c r="D120" s="169"/>
+      <c r="D120" s="158"/>
       <c r="E120" s="3" t="s">
         <v>44</v>
       </c>
@@ -33193,17 +33199,17 @@
     </row>
     <row r="126" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B126" s="112"/>
-      <c r="C126" s="169" t="s">
+      <c r="C126" s="158" t="s">
         <v>280</v>
       </c>
-      <c r="D126" s="169"/>
-      <c r="E126" s="169"/>
-      <c r="F126" s="169"/>
+      <c r="D126" s="158"/>
+      <c r="E126" s="158"/>
+      <c r="F126" s="158"/>
       <c r="K126" s="113"/>
     </row>
     <row r="127" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B127" s="112"/>
-      <c r="C127" s="168" t="s">
+      <c r="C127" s="157" t="s">
         <v>254</v>
       </c>
       <c r="D127" s="2" t="s">
@@ -33220,7 +33226,7 @@
     </row>
     <row r="128" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B128" s="112"/>
-      <c r="C128" s="168"/>
+      <c r="C128" s="157"/>
       <c r="D128" s="2" t="s">
         <v>10</v>
       </c>
@@ -33235,7 +33241,7 @@
     </row>
     <row r="129" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B129" s="112"/>
-      <c r="C129" s="168"/>
+      <c r="C129" s="157"/>
       <c r="D129" s="2" t="s">
         <v>11</v>
       </c>
@@ -33250,10 +33256,10 @@
     </row>
     <row r="130" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B130" s="112"/>
-      <c r="C130" s="161" t="s">
+      <c r="C130" s="150" t="s">
         <v>5</v>
       </c>
-      <c r="D130" s="162"/>
+      <c r="D130" s="151"/>
       <c r="E130" s="98">
         <f>+SUM(E127:E129)</f>
         <v>0.05</v>
@@ -33266,7 +33272,7 @@
     </row>
     <row r="131" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B131" s="112"/>
-      <c r="C131" s="168" t="s">
+      <c r="C131" s="157" t="s">
         <v>255</v>
       </c>
       <c r="D131" s="2" t="s">
@@ -33283,7 +33289,7 @@
     </row>
     <row r="132" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B132" s="112"/>
-      <c r="C132" s="168"/>
+      <c r="C132" s="157"/>
       <c r="D132" s="2" t="s">
         <v>10</v>
       </c>
@@ -33298,7 +33304,7 @@
     </row>
     <row r="133" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B133" s="112"/>
-      <c r="C133" s="168"/>
+      <c r="C133" s="157"/>
       <c r="D133" s="2" t="s">
         <v>11</v>
       </c>
@@ -33313,10 +33319,10 @@
     </row>
     <row r="134" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B134" s="112"/>
-      <c r="C134" s="161" t="s">
+      <c r="C134" s="150" t="s">
         <v>5</v>
       </c>
-      <c r="D134" s="162"/>
+      <c r="D134" s="151"/>
       <c r="E134" s="98">
         <f>+SUM(E131:E133)</f>
         <v>0.05</v>
@@ -33329,7 +33335,7 @@
     </row>
     <row r="135" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B135" s="112"/>
-      <c r="C135" s="168" t="s">
+      <c r="C135" s="157" t="s">
         <v>256</v>
       </c>
       <c r="D135" s="2" t="s">
@@ -33346,7 +33352,7 @@
     </row>
     <row r="136" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B136" s="112"/>
-      <c r="C136" s="168"/>
+      <c r="C136" s="157"/>
       <c r="D136" s="2" t="s">
         <v>10</v>
       </c>
@@ -33361,7 +33367,7 @@
     </row>
     <row r="137" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B137" s="112"/>
-      <c r="C137" s="168"/>
+      <c r="C137" s="157"/>
       <c r="D137" s="2" t="s">
         <v>11</v>
       </c>
@@ -33376,10 +33382,10 @@
     </row>
     <row r="138" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B138" s="112"/>
-      <c r="C138" s="161" t="s">
+      <c r="C138" s="150" t="s">
         <v>5</v>
       </c>
-      <c r="D138" s="162"/>
+      <c r="D138" s="151"/>
       <c r="E138" s="98">
         <f>+SUM(E135:E137)</f>
         <v>0.05</v>
@@ -33402,20 +33408,20 @@
     </row>
     <row r="140" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B140" s="112"/>
-      <c r="H140" s="169" t="s">
+      <c r="H140" s="158" t="s">
         <v>307</v>
       </c>
-      <c r="I140" s="169"/>
-      <c r="J140" s="169"/>
+      <c r="I140" s="158"/>
+      <c r="J140" s="158"/>
       <c r="K140" s="113"/>
     </row>
     <row r="141" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B141" s="112"/>
-      <c r="C141" s="163" t="s">
+      <c r="C141" s="152" t="s">
         <v>247</v>
       </c>
-      <c r="D141" s="164"/>
-      <c r="E141" s="165"/>
+      <c r="D141" s="153"/>
+      <c r="E141" s="154"/>
       <c r="H141" s="2" t="s">
         <v>44</v>
       </c>
@@ -33431,7 +33437,7 @@
       <c r="C142" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="D142" s="166">
+      <c r="D142" s="155">
         <v>0.05</v>
       </c>
       <c r="E142" s="27">
@@ -33456,7 +33462,7 @@
       <c r="C143" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="D143" s="166"/>
+      <c r="D143" s="155"/>
       <c r="E143" s="27">
         <f>+E101</f>
         <v>9663.2459999999992</v>
@@ -33479,7 +33485,7 @@
       <c r="C144" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="D144" s="166"/>
+      <c r="D144" s="155"/>
       <c r="E144" s="27">
         <f>+E102</f>
         <v>5239.2570000000005</v>
@@ -33502,7 +33508,7 @@
       <c r="C145" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="D145" s="166"/>
+      <c r="D145" s="155"/>
       <c r="E145" s="27">
         <f>+E103/$P$1</f>
         <v>17773.515772151903</v>
@@ -33525,7 +33531,7 @@
       <c r="C146" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="D146" s="166"/>
+      <c r="D146" s="155"/>
       <c r="E146" s="27">
         <f t="shared" ref="E146:E147" si="15">+E104/$P$1</f>
         <v>39.688810126582283</v>
@@ -33548,7 +33554,7 @@
       <c r="C147" s="2" t="s">
         <v>274</v>
       </c>
-      <c r="D147" s="166"/>
+      <c r="D147" s="155"/>
       <c r="E147" s="7">
         <f t="shared" si="15"/>
         <v>576.5266582700732</v>
@@ -33571,7 +33577,7 @@
       <c r="C148" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="D148" s="166"/>
+      <c r="D148" s="155"/>
       <c r="E148" s="7">
         <f>+E106</f>
         <v>5200.5317757272096</v>
@@ -33583,7 +33589,7 @@
       <c r="C149" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="D149" s="166"/>
+      <c r="D149" s="155"/>
       <c r="E149" s="7">
         <f>+E107</f>
         <v>5239.2570000000005</v>
@@ -33605,11 +33611,11 @@
     </row>
     <row r="152" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B152" s="112"/>
-      <c r="C152" s="163" t="s">
+      <c r="C152" s="152" t="s">
         <v>282</v>
       </c>
-      <c r="D152" s="164"/>
-      <c r="E152" s="165"/>
+      <c r="D152" s="153"/>
+      <c r="E152" s="154"/>
       <c r="K152" s="113"/>
     </row>
     <row r="153" spans="2:11" x14ac:dyDescent="0.25">
@@ -33617,7 +33623,7 @@
       <c r="C153" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="D153" s="167">
+      <c r="D153" s="156">
         <v>2.5000000000000001E-2</v>
       </c>
       <c r="E153" s="27">
@@ -33631,7 +33637,7 @@
       <c r="C154" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="D154" s="167"/>
+      <c r="D154" s="156"/>
       <c r="E154" s="27">
         <f>+E111</f>
         <v>4831.6229999999996</v>
@@ -33643,7 +33649,7 @@
       <c r="C155" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="D155" s="167"/>
+      <c r="D155" s="156"/>
       <c r="E155" s="27">
         <f>+E112</f>
         <v>2619.6285000000003</v>
@@ -33655,7 +33661,7 @@
       <c r="C156" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="D156" s="167"/>
+      <c r="D156" s="156"/>
       <c r="E156" s="27">
         <f>+E113/P1</f>
         <v>8886.7578860759513</v>
@@ -33684,10 +33690,10 @@
       <c r="K158" s="115"/>
     </row>
     <row r="164" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C164" s="174" t="s">
+      <c r="C164" s="163" t="s">
         <v>287</v>
       </c>
-      <c r="D164" s="174"/>
+      <c r="D164" s="163"/>
     </row>
     <row r="165" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C165" s="13" t="s">
@@ -33825,7 +33831,8 @@
     <col min="10" max="11" width="14.85546875" style="1" customWidth="1"/>
     <col min="12" max="12" width="13" style="1" customWidth="1"/>
     <col min="13" max="13" width="18.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="11.7109375" style="1" customWidth="1"/>
+    <col min="14" max="14" width="25" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.7109375" style="1" customWidth="1"/>
     <col min="16" max="16" width="16.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="17" max="20" width="11.42578125" style="1"/>
     <col min="21" max="21" width="18" style="1" bestFit="1" customWidth="1"/>
@@ -33857,10 +33864,10 @@
       <c r="I3" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="J3" s="224" t="s">
+      <c r="J3" s="223" t="s">
         <v>6</v>
       </c>
-      <c r="K3" s="225"/>
+      <c r="K3" s="224"/>
       <c r="L3" s="6" t="s">
         <v>7</v>
       </c>
@@ -33885,10 +33892,10 @@
       <c r="S3" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="U3" s="150" t="s">
+      <c r="U3" s="198" t="s">
         <v>245</v>
       </c>
-      <c r="V3" s="150"/>
+      <c r="V3" s="198"/>
     </row>
     <row r="4" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B4" s="16" t="s">
@@ -34098,7 +34105,7 @@
       <c r="B7" s="132" t="s">
         <v>318</v>
       </c>
-      <c r="C7" s="223">
+      <c r="C7" s="222">
         <v>46143</v>
       </c>
       <c r="D7" s="133" t="s">
@@ -34126,27 +34133,35 @@
         <f t="shared" ref="J7:J8" si="1">+F7-I7</f>
         <v>-35265.054499999998</v>
       </c>
-      <c r="K7" s="226">
+      <c r="K7" s="225">
         <f>+J7+J8</f>
         <v>-28047.695499999998</v>
       </c>
-      <c r="L7" s="199"/>
-      <c r="M7" s="135"/>
-      <c r="N7" s="136"/>
-      <c r="O7" s="136"/>
-      <c r="P7" s="199">
+      <c r="L7" s="187">
+        <v>-28048</v>
+      </c>
+      <c r="M7" s="218">
+        <v>46233</v>
+      </c>
+      <c r="N7" s="209" t="s">
+        <v>344</v>
+      </c>
+      <c r="O7" s="227">
+        <v>18</v>
+      </c>
+      <c r="P7" s="187">
         <f>+'AyD $'!F7+'AyD $'!F8</f>
         <v>-388307.41000000003</v>
       </c>
-      <c r="Q7" s="151">
+      <c r="Q7" s="212">
         <f>(+F7+F8)/P7</f>
         <v>7.6032260110616992E-2</v>
       </c>
-      <c r="R7" s="151">
+      <c r="R7" s="212">
         <f>+Q7-Q6</f>
         <v>2.2088818101272403E-2</v>
       </c>
-      <c r="S7" s="209" t="s">
+      <c r="S7" s="197" t="s">
         <v>311</v>
       </c>
       <c r="U7" s="7" t="s">
@@ -34161,8 +34176,8 @@
       <c r="B8" s="132" t="s">
         <v>319</v>
       </c>
-      <c r="C8" s="223"/>
-      <c r="D8" s="136" t="s">
+      <c r="C8" s="222"/>
+      <c r="D8" s="135" t="s">
         <v>321</v>
       </c>
       <c r="E8" s="134">
@@ -34187,21 +34202,21 @@
         <f t="shared" si="1"/>
         <v>7217.3590000000004</v>
       </c>
-      <c r="K8" s="226"/>
-      <c r="L8" s="221"/>
-      <c r="M8" s="136"/>
-      <c r="N8" s="136"/>
-      <c r="O8" s="136"/>
-      <c r="P8" s="221"/>
-      <c r="Q8" s="152"/>
-      <c r="R8" s="152"/>
-      <c r="S8" s="227"/>
+      <c r="K8" s="225"/>
+      <c r="L8" s="210"/>
+      <c r="M8" s="219"/>
+      <c r="N8" s="206"/>
+      <c r="O8" s="228"/>
+      <c r="P8" s="210"/>
+      <c r="Q8" s="213"/>
+      <c r="R8" s="213"/>
+      <c r="S8" s="226"/>
       <c r="U8" s="7" t="s">
         <v>7</v>
       </c>
       <c r="V8" s="7">
         <f>+L10</f>
-        <v>57834.413499999995</v>
+        <v>29786.413499999995</v>
       </c>
     </row>
     <row r="10" spans="2:22" x14ac:dyDescent="0.25">
@@ -34229,18 +34244,18 @@
       <c r="K10" s="22"/>
       <c r="L10" s="22">
         <f t="shared" si="2"/>
-        <v>57834.413499999995</v>
+        <v>29786.413499999995</v>
       </c>
       <c r="M10" s="22">
         <f t="shared" si="2"/>
-        <v>137701</v>
+        <v>183934</v>
       </c>
       <c r="N10" s="22"/>
       <c r="O10" s="22"/>
       <c r="R10" s="19"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="12">
     <mergeCell ref="U3:V3"/>
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="J3:K3"/>
@@ -34250,6 +34265,9 @@
     <mergeCell ref="R7:R8"/>
     <mergeCell ref="S7:S8"/>
     <mergeCell ref="L7:L8"/>
+    <mergeCell ref="O7:O8"/>
+    <mergeCell ref="M7:M8"/>
+    <mergeCell ref="N7:N8"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -34288,39 +34306,39 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B2" s="202" t="s">
+      <c r="B2" s="190" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="202" t="s">
+      <c r="C2" s="190" t="s">
         <v>64</v>
       </c>
-      <c r="D2" s="172" t="s">
+      <c r="D2" s="161" t="s">
         <v>84</v>
       </c>
-      <c r="E2" s="207"/>
-      <c r="F2" s="207"/>
-      <c r="G2" s="207"/>
-      <c r="H2" s="207"/>
-      <c r="I2" s="207"/>
-      <c r="J2" s="207"/>
-      <c r="K2" s="207"/>
-      <c r="L2" s="207"/>
-      <c r="M2" s="207"/>
-      <c r="N2" s="169" t="s">
+      <c r="E2" s="195"/>
+      <c r="F2" s="195"/>
+      <c r="G2" s="195"/>
+      <c r="H2" s="195"/>
+      <c r="I2" s="195"/>
+      <c r="J2" s="195"/>
+      <c r="K2" s="195"/>
+      <c r="L2" s="195"/>
+      <c r="M2" s="195"/>
+      <c r="N2" s="158" t="s">
         <v>85</v>
       </c>
-      <c r="O2" s="169"/>
-      <c r="P2" s="169"/>
-      <c r="Q2" s="169"/>
-      <c r="R2" s="169"/>
-      <c r="S2" s="169"/>
-      <c r="T2" s="169"/>
-      <c r="U2" s="169"/>
-      <c r="V2" s="169"/>
+      <c r="O2" s="158"/>
+      <c r="P2" s="158"/>
+      <c r="Q2" s="158"/>
+      <c r="R2" s="158"/>
+      <c r="S2" s="158"/>
+      <c r="T2" s="158"/>
+      <c r="U2" s="158"/>
+      <c r="V2" s="158"/>
     </row>
     <row r="3" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B3" s="202"/>
-      <c r="C3" s="202"/>
+      <c r="B3" s="190"/>
+      <c r="C3" s="190"/>
       <c r="D3" s="56" t="s">
         <v>3</v>
       </c>
@@ -35976,11 +35994,11 @@
         <f>+N34-Q34-R34-S34-T34-U34-L34</f>
         <v>-6171.5616950964513</v>
       </c>
-      <c r="W34" s="215">
+      <c r="W34" s="204">
         <f>+V34+V35+V36+V37</f>
         <v>78154.97</v>
       </c>
-      <c r="X34" s="177" t="s">
+      <c r="X34" s="166" t="s">
         <v>195</v>
       </c>
     </row>
@@ -36024,8 +36042,8 @@
         <f>+N35-Q35-R35-S35-T35-U35</f>
         <v>84326.531695096448</v>
       </c>
-      <c r="W35" s="177"/>
-      <c r="X35" s="177"/>
+      <c r="W35" s="166"/>
+      <c r="X35" s="166"/>
     </row>
     <row r="36" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B36" s="15" t="s">
@@ -36066,8 +36084,8 @@
         <f>+N36-T36</f>
         <v>-527.4400463149974</v>
       </c>
-      <c r="W36" s="177"/>
-      <c r="X36" s="177"/>
+      <c r="W36" s="166"/>
+      <c r="X36" s="166"/>
     </row>
     <row r="37" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B37" s="15" t="s">
@@ -36109,8 +36127,8 @@
         <f>+N37-T37</f>
         <v>527.4400463149974</v>
       </c>
-      <c r="W37" s="177"/>
-      <c r="X37" s="177"/>
+      <c r="W37" s="166"/>
+      <c r="X37" s="166"/>
     </row>
     <row r="38" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B38" s="15" t="s">
@@ -36274,11 +36292,11 @@
         <f>+'Básico USD CIF'!N5+'AYD USD CIF'!K6+'AYD USD CIF'!K7</f>
         <v>-161.83360646833864</v>
       </c>
-      <c r="W40" s="215">
+      <c r="W40" s="204">
         <f>+V40+V41</f>
         <v>1887.3837500000004</v>
       </c>
-      <c r="X40" s="177" t="s">
+      <c r="X40" s="166" t="s">
         <v>195</v>
       </c>
     </row>
@@ -36331,8 +36349,8 @@
         <f>+'AYD USD Plaza '!K6+'AYD USD Plaza '!K7</f>
         <v>2049.2173564683389</v>
       </c>
-      <c r="W41" s="215"/>
-      <c r="X41" s="177"/>
+      <c r="W41" s="204"/>
+      <c r="X41" s="166"/>
     </row>
     <row r="42" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B42" s="12" t="s">
@@ -36538,11 +36556,11 @@
         <f>+N45-Q45-R45-S45-T45-U45</f>
         <v>9079.4637500000008</v>
       </c>
-      <c r="W45" s="228">
+      <c r="W45" s="229">
         <f>+V45+V46+V47</f>
         <v>9079.463749999999</v>
       </c>
-      <c r="X45" s="177" t="s">
+      <c r="X45" s="166" t="s">
         <v>195</v>
       </c>
     </row>
@@ -36586,8 +36604,8 @@
         <f t="shared" ref="V46:V47" si="1">+N46-Q46-R46-S46-T46-U46</f>
         <v>9857.7035730159078</v>
       </c>
-      <c r="W46" s="228"/>
-      <c r="X46" s="177"/>
+      <c r="W46" s="229"/>
+      <c r="X46" s="166"/>
     </row>
     <row r="47" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B47" s="12" t="s">
@@ -36628,15 +36646,15 @@
         <f t="shared" si="1"/>
         <v>-9857.7035730159078</v>
       </c>
-      <c r="W47" s="228"/>
-      <c r="X47" s="177"/>
+      <c r="W47" s="229"/>
+      <c r="X47" s="166"/>
     </row>
     <row r="48" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B48" s="12" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D48" s="7">
         <f>+'Básico $'!F23+AP!F22</f>
@@ -36693,7 +36711,7 @@
         <v>311</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D49" s="7">
         <f>+'AP Adicionales'!F7+'AP Adicionales'!F8</f>
@@ -36730,7 +36748,7 @@
       <c r="U49" s="7"/>
       <c r="V49" s="7"/>
       <c r="W49" s="1" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="50" spans="2:24" x14ac:dyDescent="0.25">
@@ -36738,7 +36756,7 @@
         <v>124</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D50" s="7"/>
       <c r="E50" s="7"/>
@@ -36792,7 +36810,7 @@
         <v>125</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="D51" s="7"/>
       <c r="E51" s="7"/>
@@ -36813,11 +36831,11 @@
       <c r="T51" s="7"/>
       <c r="U51" s="7"/>
       <c r="V51" s="7"/>
-      <c r="W51" s="228">
+      <c r="W51" s="229">
         <f>+V51+V52+V53</f>
         <v>0</v>
       </c>
-      <c r="X51" s="177" t="s">
+      <c r="X51" s="166" t="s">
         <v>195</v>
       </c>
     </row>
@@ -36826,7 +36844,7 @@
         <v>126</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="D52" s="7"/>
       <c r="E52" s="7"/>
@@ -36847,15 +36865,15 @@
       <c r="T52" s="7"/>
       <c r="U52" s="7"/>
       <c r="V52" s="7"/>
-      <c r="W52" s="228"/>
-      <c r="X52" s="177"/>
+      <c r="W52" s="229"/>
+      <c r="X52" s="166"/>
     </row>
     <row r="53" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B53" s="12" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D53" s="7"/>
       <c r="E53" s="7"/>
@@ -36876,8 +36894,8 @@
       <c r="T53" s="7"/>
       <c r="U53" s="7"/>
       <c r="V53" s="7"/>
-      <c r="W53" s="228"/>
-      <c r="X53" s="177"/>
+      <c r="W53" s="229"/>
+      <c r="X53" s="166"/>
     </row>
   </sheetData>
   <autoFilter ref="B3:M3" xr:uid="{441EF1EB-ECA0-4462-8CF3-F31A7CAFCD96}">
@@ -36927,13 +36945,13 @@
         <v>291</v>
       </c>
       <c r="C3" s="4" t="s">
+        <v>322</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>323</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="E3" s="4" t="s">
         <v>324</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>325</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>6</v>
@@ -37081,12 +37099,12 @@
     </row>
     <row r="2" spans="2:37" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
-        <v>335</v>
-      </c>
-      <c r="AK2" s="138"/>
+        <v>334</v>
+      </c>
+      <c r="AK2" s="137"/>
     </row>
     <row r="3" spans="2:37" x14ac:dyDescent="0.25">
-      <c r="AK3" s="138"/>
+      <c r="AK3" s="137"/>
     </row>
     <row r="4" spans="2:37" x14ac:dyDescent="0.25">
       <c r="B4" s="88" t="s">
@@ -37100,10 +37118,10 @@
       <c r="M5" s="88"/>
     </row>
     <row r="6" spans="2:37" s="34" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="188" t="s">
+      <c r="B6" s="177" t="s">
         <v>64</v>
       </c>
-      <c r="C6" s="188"/>
+      <c r="C6" s="177"/>
       <c r="D6" s="46" t="s">
         <v>63</v>
       </c>
@@ -37175,7 +37193,7 @@
       <c r="AI6"/>
     </row>
     <row r="7" spans="2:37" x14ac:dyDescent="0.25">
-      <c r="B7" s="176" t="s">
+      <c r="B7" s="165" t="s">
         <v>70</v>
       </c>
       <c r="C7" s="33" t="s">
@@ -37184,12 +37202,12 @@
       <c r="D7" s="30">
         <v>446784590</v>
       </c>
-      <c r="E7" s="189">
+      <c r="E7" s="178">
         <f>+D7*$F$6</f>
         <v>8935691.8000000007</v>
       </c>
-      <c r="F7" s="189"/>
-      <c r="G7" s="190">
+      <c r="F7" s="178"/>
+      <c r="G7" s="179">
         <v>45805</v>
       </c>
       <c r="H7" s="30">
@@ -37204,7 +37222,7 @@
         <f>+E7/I7</f>
         <v>2.1697976243534034E-2</v>
       </c>
-      <c r="K7" s="187" t="s">
+      <c r="K7" s="176" t="s">
         <v>68</v>
       </c>
       <c r="M7" s="33" t="s">
@@ -37259,19 +37277,19 @@
       <c r="AD7" s="124"/>
     </row>
     <row r="8" spans="2:37" x14ac:dyDescent="0.25">
-      <c r="B8" s="177"/>
+      <c r="B8" s="166"/>
       <c r="C8" s="33" t="s">
         <v>66</v>
       </c>
       <c r="D8" s="30">
         <v>637404</v>
       </c>
-      <c r="E8" s="189">
+      <c r="E8" s="178">
         <f t="shared" ref="E8:E9" si="0">+D8*$F$6</f>
         <v>12748.08</v>
       </c>
-      <c r="F8" s="189"/>
-      <c r="G8" s="190"/>
+      <c r="F8" s="178"/>
+      <c r="G8" s="179"/>
       <c r="H8" s="37">
         <v>0</v>
       </c>
@@ -37283,7 +37301,7 @@
         <f t="shared" ref="J8:J9" si="2">+E8/I8</f>
         <v>0.02</v>
       </c>
-      <c r="K8" s="187"/>
+      <c r="K8" s="176"/>
       <c r="M8" s="33" t="s">
         <v>242</v>
       </c>
@@ -37336,19 +37354,19 @@
       <c r="AD8" s="124"/>
     </row>
     <row r="9" spans="2:37" x14ac:dyDescent="0.25">
-      <c r="B9" s="177"/>
+      <c r="B9" s="166"/>
       <c r="C9" s="33" t="s">
         <v>67</v>
       </c>
       <c r="D9" s="30">
         <v>451303</v>
       </c>
-      <c r="E9" s="189">
+      <c r="E9" s="178">
         <f t="shared" si="0"/>
         <v>9026.06</v>
       </c>
-      <c r="F9" s="189"/>
-      <c r="G9" s="190"/>
+      <c r="F9" s="178"/>
+      <c r="G9" s="179"/>
       <c r="H9" s="37">
         <v>0</v>
       </c>
@@ -37360,7 +37378,7 @@
         <f t="shared" si="2"/>
         <v>0.02</v>
       </c>
-      <c r="K9" s="187"/>
+      <c r="K9" s="176"/>
       <c r="M9" s="33" t="s">
         <v>67</v>
       </c>
@@ -37424,10 +37442,10 @@
       <c r="K10" s="41"/>
     </row>
     <row r="11" spans="2:37" x14ac:dyDescent="0.25">
-      <c r="B11" s="175" t="s">
+      <c r="B11" s="164" t="s">
         <v>64</v>
       </c>
-      <c r="C11" s="175"/>
+      <c r="C11" s="164"/>
       <c r="D11" s="38" t="s">
         <v>63</v>
       </c>
@@ -37454,7 +37472,7 @@
       </c>
     </row>
     <row r="12" spans="2:37" x14ac:dyDescent="0.25">
-      <c r="B12" s="176" t="s">
+      <c r="B12" s="165" t="s">
         <v>114</v>
       </c>
       <c r="C12" s="33" t="s">
@@ -37463,12 +37481,12 @@
       <c r="D12" s="30">
         <v>446784590</v>
       </c>
-      <c r="E12" s="178">
+      <c r="E12" s="167">
         <f>+D12*$F$11</f>
         <v>6701768.8499999996</v>
       </c>
-      <c r="F12" s="178"/>
-      <c r="G12" s="192">
+      <c r="F12" s="167"/>
+      <c r="G12" s="181">
         <v>45975</v>
       </c>
       <c r="H12" s="30">
@@ -37482,24 +37500,24 @@
       <c r="J12" s="39">
         <v>2.2324E-2</v>
       </c>
-      <c r="K12" s="187" t="s">
+      <c r="K12" s="176" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="13" spans="2:37" x14ac:dyDescent="0.25">
-      <c r="B13" s="177"/>
+      <c r="B13" s="166"/>
       <c r="C13" s="33" t="s">
         <v>66</v>
       </c>
       <c r="D13" s="30">
         <v>637404</v>
       </c>
-      <c r="E13" s="189">
+      <c r="E13" s="178">
         <f t="shared" ref="E13:E14" si="6">+D13*$F$11</f>
         <v>9561.06</v>
       </c>
-      <c r="F13" s="189"/>
-      <c r="G13" s="180"/>
+      <c r="F13" s="178"/>
+      <c r="G13" s="169"/>
       <c r="H13" s="37">
         <v>0</v>
       </c>
@@ -37511,22 +37529,22 @@
         <f t="shared" ref="J13:J14" si="8">+E13/I13</f>
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="K13" s="187"/>
+      <c r="K13" s="176"/>
     </row>
     <row r="14" spans="2:37" x14ac:dyDescent="0.25">
-      <c r="B14" s="177"/>
+      <c r="B14" s="166"/>
       <c r="C14" s="33" t="s">
         <v>67</v>
       </c>
       <c r="D14" s="30">
         <v>451303</v>
       </c>
-      <c r="E14" s="189">
+      <c r="E14" s="178">
         <f t="shared" si="6"/>
         <v>6769.5450000000001</v>
       </c>
-      <c r="F14" s="189"/>
-      <c r="G14" s="180"/>
+      <c r="F14" s="178"/>
+      <c r="G14" s="169"/>
       <c r="H14" s="37">
         <v>0</v>
       </c>
@@ -37538,13 +37556,13 @@
         <f t="shared" si="8"/>
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="K14" s="187"/>
+      <c r="K14" s="176"/>
     </row>
     <row r="16" spans="2:37" x14ac:dyDescent="0.25">
-      <c r="B16" s="175" t="s">
+      <c r="B16" s="164" t="s">
         <v>64</v>
       </c>
-      <c r="C16" s="175"/>
+      <c r="C16" s="164"/>
       <c r="D16" s="38" t="s">
         <v>63</v>
       </c>
@@ -37571,7 +37589,7 @@
       </c>
     </row>
     <row r="17" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B17" s="176" t="s">
+      <c r="B17" s="165" t="s">
         <v>115</v>
       </c>
       <c r="C17" s="33" t="s">
@@ -37580,12 +37598,12 @@
       <c r="D17" s="30">
         <v>446784590</v>
       </c>
-      <c r="E17" s="178">
+      <c r="E17" s="167">
         <f>+D17*$F$11</f>
         <v>6701768.8499999996</v>
       </c>
-      <c r="F17" s="178"/>
-      <c r="G17" s="191">
+      <c r="F17" s="167"/>
+      <c r="G17" s="180">
         <v>46101</v>
       </c>
       <c r="H17" s="30">
@@ -37598,24 +37616,24 @@
       <c r="J17" s="71">
         <v>2.8398E-2</v>
       </c>
-      <c r="K17" s="180">
+      <c r="K17" s="169">
         <v>102</v>
       </c>
     </row>
     <row r="18" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B18" s="177"/>
+      <c r="B18" s="166"/>
       <c r="C18" s="33" t="s">
         <v>66</v>
       </c>
       <c r="D18" s="30">
         <v>637404</v>
       </c>
-      <c r="E18" s="189">
+      <c r="E18" s="178">
         <f t="shared" ref="E18:E19" si="9">+D18*$F$11</f>
         <v>9561.06</v>
       </c>
-      <c r="F18" s="189"/>
-      <c r="G18" s="177"/>
+      <c r="F18" s="178"/>
+      <c r="G18" s="166"/>
       <c r="H18" s="37">
         <f>+'Básico USD Plaza'!F4</f>
         <v>17074.7</v>
@@ -37628,22 +37646,22 @@
         <f t="shared" ref="J18:J19" si="11">+E18/I18</f>
         <v>1.5412878288999083E-2</v>
       </c>
-      <c r="K18" s="180"/>
+      <c r="K18" s="169"/>
     </row>
     <row r="19" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B19" s="177"/>
+      <c r="B19" s="166"/>
       <c r="C19" s="33" t="s">
         <v>67</v>
       </c>
       <c r="D19" s="30">
         <v>451303</v>
       </c>
-      <c r="E19" s="189">
+      <c r="E19" s="178">
         <f t="shared" si="9"/>
         <v>6769.5450000000001</v>
       </c>
-      <c r="F19" s="189"/>
-      <c r="G19" s="177"/>
+      <c r="F19" s="178"/>
+      <c r="G19" s="166"/>
       <c r="H19" s="37">
         <v>0</v>
       </c>
@@ -37655,40 +37673,40 @@
         <f t="shared" si="11"/>
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="K19" s="180"/>
+      <c r="K19" s="169"/>
     </row>
     <row r="53" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B53" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="55" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B55" s="88" t="s">
         <v>243</v>
       </c>
-      <c r="M55" s="141" t="s">
-        <v>343</v>
-      </c>
-      <c r="N55" s="141">
+      <c r="M55" s="140" t="s">
+        <v>342</v>
+      </c>
+      <c r="N55" s="140">
         <v>38.792000000000002</v>
       </c>
     </row>
     <row r="57" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B57" s="188" t="s">
+      <c r="B57" s="177" t="s">
         <v>64</v>
       </c>
-      <c r="C57" s="188"/>
+      <c r="C57" s="177"/>
       <c r="D57" s="46" t="s">
         <v>63</v>
       </c>
       <c r="E57" s="38" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F57" s="69">
         <v>0.02</v>
       </c>
       <c r="G57" s="47" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="H57" s="36" t="s">
         <v>167</v>
@@ -37704,7 +37722,7 @@
       </c>
     </row>
     <row r="58" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B58" s="176" t="s">
+      <c r="B58" s="165" t="s">
         <v>70</v>
       </c>
       <c r="C58" s="33" t="s">
@@ -37713,64 +37731,64 @@
       <c r="D58" s="30">
         <v>166552456</v>
       </c>
-      <c r="E58" s="189">
+      <c r="E58" s="178">
         <f>D58*$F$57</f>
         <v>3331049.12</v>
       </c>
-      <c r="F58" s="189"/>
-      <c r="G58" s="190" t="s">
-        <v>342</v>
-      </c>
-      <c r="H58" s="181">
+      <c r="F58" s="178"/>
+      <c r="G58" s="179" t="s">
+        <v>341</v>
+      </c>
+      <c r="H58" s="170">
         <v>30437309</v>
       </c>
-      <c r="I58" s="181">
+      <c r="I58" s="170">
         <f>+D58+(D59*TC+D60*TC)-H58</f>
         <v>156254277.58560002</v>
       </c>
-      <c r="J58" s="184">
+      <c r="J58" s="173">
         <f>(E58+(E59*TC+E60*TC))/I58</f>
         <v>2.3895868896558776E-2</v>
       </c>
-      <c r="K58" s="187"/>
+      <c r="K58" s="176"/>
     </row>
     <row r="59" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B59" s="177"/>
+      <c r="B59" s="166"/>
       <c r="C59" s="33" t="s">
         <v>66</v>
       </c>
       <c r="D59" s="30">
         <v>294444.5</v>
       </c>
-      <c r="E59" s="189">
+      <c r="E59" s="178">
         <f t="shared" ref="E59:E60" si="12">D59*$F$57</f>
         <v>5888.89</v>
       </c>
-      <c r="F59" s="189"/>
-      <c r="G59" s="190"/>
-      <c r="H59" s="182"/>
-      <c r="I59" s="182"/>
-      <c r="J59" s="185"/>
-      <c r="K59" s="187"/>
+      <c r="F59" s="178"/>
+      <c r="G59" s="179"/>
+      <c r="H59" s="171"/>
+      <c r="I59" s="171"/>
+      <c r="J59" s="174"/>
+      <c r="K59" s="176"/>
     </row>
     <row r="60" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B60" s="177"/>
+      <c r="B60" s="166"/>
       <c r="C60" s="33" t="s">
         <v>67</v>
       </c>
       <c r="D60" s="30">
         <v>224712.30000000005</v>
       </c>
-      <c r="E60" s="189">
+      <c r="E60" s="178">
         <f t="shared" si="12"/>
         <v>4494.246000000001</v>
       </c>
-      <c r="F60" s="189"/>
-      <c r="G60" s="190"/>
-      <c r="H60" s="183"/>
-      <c r="I60" s="183"/>
-      <c r="J60" s="186"/>
-      <c r="K60" s="187"/>
+      <c r="F60" s="178"/>
+      <c r="G60" s="179"/>
+      <c r="H60" s="172"/>
+      <c r="I60" s="172"/>
+      <c r="J60" s="175"/>
+      <c r="K60" s="176"/>
     </row>
     <row r="61" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B61" s="43"/>
@@ -37778,35 +37796,35 @@
       <c r="E61" s="44"/>
       <c r="F61" s="44"/>
       <c r="G61" s="40"/>
-      <c r="H61" s="144"/>
-      <c r="I61" s="145"/>
-      <c r="J61" s="146"/>
+      <c r="H61" s="143"/>
+      <c r="I61" s="144"/>
+      <c r="J61" s="145"/>
       <c r="K61" s="41"/>
     </row>
     <row r="62" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B62" s="175" t="s">
+      <c r="B62" s="164" t="s">
         <v>64</v>
       </c>
-      <c r="C62" s="175"/>
+      <c r="C62" s="164"/>
       <c r="D62" s="38" t="s">
         <v>63</v>
       </c>
       <c r="E62" s="38" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F62" s="70">
         <v>1.4999999999999999E-2</v>
       </c>
       <c r="G62" s="47" t="s">
-        <v>336</v>
-      </c>
-      <c r="H62" s="147" t="s">
+        <v>335</v>
+      </c>
+      <c r="H62" s="146" t="s">
         <v>167</v>
       </c>
-      <c r="I62" s="147" t="s">
+      <c r="I62" s="146" t="s">
         <v>69</v>
       </c>
-      <c r="J62" s="147" t="s">
+      <c r="J62" s="146" t="s">
         <v>72</v>
       </c>
       <c r="K62" s="35" t="s">
@@ -37814,7 +37832,7 @@
       </c>
     </row>
     <row r="63" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B63" s="176" t="s">
+      <c r="B63" s="165" t="s">
         <v>114</v>
       </c>
       <c r="C63" s="33" t="s">
@@ -37823,94 +37841,94 @@
       <c r="D63" s="30">
         <v>166552456</v>
       </c>
-      <c r="E63" s="178">
+      <c r="E63" s="167">
         <f>+D63*$F$62</f>
         <v>2498286.84</v>
       </c>
-      <c r="F63" s="178"/>
-      <c r="G63" s="179">
+      <c r="F63" s="167"/>
+      <c r="G63" s="168">
         <v>46357</v>
       </c>
-      <c r="H63" s="181">
+      <c r="H63" s="170">
         <v>69480418</v>
       </c>
-      <c r="I63" s="181">
+      <c r="I63" s="170">
         <f>+D63+(D64*TC+D65*TC)-H63</f>
         <v>117211168.58560002</v>
       </c>
-      <c r="J63" s="184">
+      <c r="J63" s="173">
         <f>(E63+(E64*TC+E65*TC))/I63</f>
         <v>2.3891697630664524E-2</v>
       </c>
-      <c r="K63" s="187"/>
+      <c r="K63" s="176"/>
     </row>
     <row r="64" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B64" s="177"/>
+      <c r="B64" s="166"/>
       <c r="C64" s="33" t="s">
         <v>66</v>
       </c>
       <c r="D64" s="30">
         <v>294444.5</v>
       </c>
-      <c r="E64" s="178">
+      <c r="E64" s="167">
         <f t="shared" ref="E64:E65" si="13">+D64*$F$62</f>
         <v>4416.6674999999996</v>
       </c>
-      <c r="F64" s="178"/>
-      <c r="G64" s="180"/>
-      <c r="H64" s="182"/>
-      <c r="I64" s="182"/>
-      <c r="J64" s="185"/>
-      <c r="K64" s="187"/>
+      <c r="F64" s="167"/>
+      <c r="G64" s="169"/>
+      <c r="H64" s="171"/>
+      <c r="I64" s="171"/>
+      <c r="J64" s="174"/>
+      <c r="K64" s="176"/>
     </row>
     <row r="65" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B65" s="177"/>
+      <c r="B65" s="166"/>
       <c r="C65" s="33" t="s">
         <v>67</v>
       </c>
       <c r="D65" s="30">
         <v>224712.30000000005</v>
       </c>
-      <c r="E65" s="178">
+      <c r="E65" s="167">
         <f t="shared" si="13"/>
         <v>3370.6845000000008</v>
       </c>
-      <c r="F65" s="178"/>
-      <c r="G65" s="180"/>
-      <c r="H65" s="183"/>
-      <c r="I65" s="183"/>
-      <c r="J65" s="186"/>
-      <c r="K65" s="187"/>
+      <c r="F65" s="167"/>
+      <c r="G65" s="169"/>
+      <c r="H65" s="172"/>
+      <c r="I65" s="172"/>
+      <c r="J65" s="175"/>
+      <c r="K65" s="176"/>
     </row>
     <row r="66" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="H66" s="148"/>
-      <c r="I66" s="148"/>
-      <c r="J66" s="148"/>
+      <c r="H66" s="147"/>
+      <c r="I66" s="147"/>
+      <c r="J66" s="147"/>
     </row>
     <row r="67" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B67" s="175" t="s">
+      <c r="B67" s="164" t="s">
         <v>64</v>
       </c>
-      <c r="C67" s="175"/>
+      <c r="C67" s="164"/>
       <c r="D67" s="38" t="s">
         <v>63</v>
       </c>
       <c r="E67" s="38" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F67" s="70">
         <v>1.4999999999999999E-2</v>
       </c>
       <c r="G67" s="47" t="s">
-        <v>336</v>
-      </c>
-      <c r="H67" s="147" t="s">
+        <v>335</v>
+      </c>
+      <c r="H67" s="146" t="s">
         <v>167</v>
       </c>
-      <c r="I67" s="147" t="s">
+      <c r="I67" s="146" t="s">
         <v>69</v>
       </c>
-      <c r="J67" s="147" t="s">
+      <c r="J67" s="146" t="s">
         <v>72</v>
       </c>
       <c r="K67" s="35" t="s">
@@ -37918,7 +37936,7 @@
       </c>
     </row>
     <row r="68" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B68" s="176" t="s">
+      <c r="B68" s="165" t="s">
         <v>115</v>
       </c>
       <c r="C68" s="33" t="s">
@@ -37927,95 +37945,95 @@
       <c r="D68" s="30">
         <v>166552456</v>
       </c>
-      <c r="E68" s="178">
+      <c r="E68" s="167">
         <f>+D68*$F$67</f>
         <v>2498286.84</v>
       </c>
-      <c r="F68" s="178"/>
-      <c r="G68" s="179">
+      <c r="F68" s="167"/>
+      <c r="G68" s="168">
         <v>46508</v>
       </c>
-      <c r="H68" s="181">
+      <c r="H68" s="170">
         <v>133306761</v>
       </c>
-      <c r="I68" s="181">
+      <c r="I68" s="170">
         <f>+D68+(D69*TC+D70*TC)-H68</f>
         <v>53384825.585600019</v>
       </c>
-      <c r="J68" s="184">
+      <c r="J68" s="173">
         <f>(E68+(E69*TC+E70*TC))/I68</f>
         <v>5.2456363171848042E-2</v>
       </c>
-      <c r="K68" s="180"/>
+      <c r="K68" s="169"/>
     </row>
     <row r="69" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B69" s="177"/>
+      <c r="B69" s="166"/>
       <c r="C69" s="33" t="s">
         <v>66</v>
       </c>
       <c r="D69" s="30">
         <v>294444.5</v>
       </c>
-      <c r="E69" s="178">
+      <c r="E69" s="167">
         <f t="shared" ref="E69:E70" si="14">+D69*$F$67</f>
         <v>4416.6674999999996</v>
       </c>
-      <c r="F69" s="178"/>
-      <c r="G69" s="180"/>
-      <c r="H69" s="182"/>
-      <c r="I69" s="182"/>
-      <c r="J69" s="185"/>
-      <c r="K69" s="180"/>
+      <c r="F69" s="167"/>
+      <c r="G69" s="169"/>
+      <c r="H69" s="171"/>
+      <c r="I69" s="171"/>
+      <c r="J69" s="174"/>
+      <c r="K69" s="169"/>
     </row>
     <row r="70" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B70" s="177"/>
+      <c r="B70" s="166"/>
       <c r="C70" s="33" t="s">
         <v>67</v>
       </c>
       <c r="D70" s="30">
         <v>224712.30000000005</v>
       </c>
-      <c r="E70" s="178">
+      <c r="E70" s="167">
         <f t="shared" si="14"/>
         <v>3370.6845000000008</v>
       </c>
-      <c r="F70" s="178"/>
-      <c r="G70" s="180"/>
-      <c r="H70" s="183"/>
-      <c r="I70" s="183"/>
-      <c r="J70" s="186"/>
-      <c r="K70" s="180"/>
+      <c r="F70" s="167"/>
+      <c r="G70" s="169"/>
+      <c r="H70" s="172"/>
+      <c r="I70" s="172"/>
+      <c r="J70" s="175"/>
+      <c r="K70" s="169"/>
     </row>
     <row r="74" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D74" s="33" t="s">
-        <v>338</v>
-      </c>
-      <c r="E74" s="143">
+        <v>337</v>
+      </c>
+      <c r="E74" s="142">
         <f>+E58+E59*TC+E60*TC</f>
         <v>3733831.731712</v>
       </c>
     </row>
     <row r="75" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D75" s="33" t="s">
-        <v>339</v>
-      </c>
-      <c r="E75" s="143">
+        <v>338</v>
+      </c>
+      <c r="E75" s="142">
         <f>+E63+E64*TC+E65*TC</f>
         <v>2800373.7987839999</v>
       </c>
     </row>
     <row r="76" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D76" s="33" t="s">
-        <v>340</v>
-      </c>
-      <c r="E76" s="143">
+        <v>339</v>
+      </c>
+      <c r="E76" s="142">
         <f>+E68+E70*TC+E69*TC</f>
         <v>2800373.7987839999</v>
       </c>
     </row>
     <row r="83" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B83" s="42"/>
-      <c r="C83" s="139"/>
+      <c r="C83" s="138"/>
     </row>
     <row r="84" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B84" s="42"/>
@@ -38024,19 +38042,19 @@
       <c r="B85" s="42"/>
     </row>
     <row r="87" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C87" s="139"/>
+      <c r="C87" s="138"/>
     </row>
     <row r="88" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B88" s="140"/>
+      <c r="B88" s="139"/>
     </row>
     <row r="89" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B89" s="139"/>
+      <c r="B89" s="138"/>
     </row>
     <row r="92" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B92" s="139"/>
+      <c r="B92" s="138"/>
     </row>
     <row r="93" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B93" s="142"/>
+      <c r="B93" s="141"/>
     </row>
   </sheetData>
   <mergeCells count="51">
@@ -38161,26 +38179,26 @@
       </c>
     </row>
     <row r="2" spans="2:51" x14ac:dyDescent="0.25">
-      <c r="AB2" s="193" t="s">
+      <c r="AB2" s="149" t="s">
         <v>269</v>
       </c>
-      <c r="AC2" s="193"/>
-      <c r="AG2" s="193" t="s">
+      <c r="AC2" s="149"/>
+      <c r="AG2" s="149" t="s">
         <v>4</v>
       </c>
-      <c r="AH2" s="193"/>
-      <c r="AM2" s="193" t="s">
+      <c r="AH2" s="149"/>
+      <c r="AM2" s="149" t="s">
         <v>259</v>
       </c>
-      <c r="AN2" s="193"/>
-      <c r="AR2" s="193" t="s">
+      <c r="AN2" s="149"/>
+      <c r="AR2" s="149" t="s">
         <v>258</v>
       </c>
-      <c r="AS2" s="193"/>
-      <c r="AX2" s="193" t="s">
+      <c r="AS2" s="149"/>
+      <c r="AX2" s="149" t="s">
         <v>262</v>
       </c>
-      <c r="AY2" s="193"/>
+      <c r="AY2" s="149"/>
     </row>
     <row r="3" spans="2:51" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
@@ -38246,10 +38264,10 @@
       <c r="V3" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="X3" s="193" t="s">
+      <c r="X3" s="149" t="s">
         <v>245</v>
       </c>
-      <c r="Y3" s="193"/>
+      <c r="Y3" s="149"/>
       <c r="AB3" s="102" t="s">
         <v>244</v>
       </c>
@@ -39454,7 +39472,7 @@
         <f t="shared" si="17"/>
         <v>310621.22500000003</v>
       </c>
-      <c r="N19" s="149">
+      <c r="N19" s="148">
         <f t="shared" si="6"/>
         <v>10946018.622322002</v>
       </c>
@@ -39530,7 +39548,7 @@
         <f t="shared" si="17"/>
         <v>374962.91425000003</v>
       </c>
-      <c r="N20" s="149">
+      <c r="N20" s="148">
         <f t="shared" si="6"/>
         <v>12787435.257250601</v>
       </c>
@@ -39605,7 +39623,7 @@
         <f t="shared" si="17"/>
         <v>307383.45650000003</v>
       </c>
-      <c r="N21" s="149">
+      <c r="N21" s="148">
         <f t="shared" si="6"/>
         <v>10482759.493710799</v>
       </c>
@@ -39680,7 +39698,7 @@
         <f t="shared" si="17"/>
         <v>374421.16400000005</v>
       </c>
-      <c r="N22" s="149">
+      <c r="N22" s="148">
         <f t="shared" si="6"/>
         <v>12768959.840124801</v>
       </c>
@@ -39720,7 +39738,7 @@
         <v>46174</v>
       </c>
       <c r="D23" s="66" t="s">
-        <v>322</v>
+        <v>343</v>
       </c>
       <c r="E23" s="9">
         <v>46203</v>
@@ -39756,7 +39774,7 @@
         <f t="shared" si="17"/>
         <v>376055.32500000001</v>
       </c>
-      <c r="N23" s="149">
+      <c r="N23" s="148">
         <f>+F23-I23-J23-K23-L23-M23</f>
         <v>12824689.959539998</v>
       </c>
@@ -39781,7 +39799,9 @@
       <c r="T23" s="2" t="s">
         <v>309</v>
       </c>
-      <c r="U23" s="12"/>
+      <c r="U23" s="12">
+        <v>18</v>
+      </c>
       <c r="V23" s="28" t="s">
         <v>310</v>
       </c>
@@ -39989,7 +40009,7 @@
       <c r="M42" s="10"/>
       <c r="N42" s="10"/>
       <c r="O42" s="10"/>
-      <c r="P42" s="137"/>
+      <c r="P42" s="136"/>
       <c r="S42" s="1"/>
     </row>
     <row r="43" spans="1:19" x14ac:dyDescent="0.25">
@@ -40385,26 +40405,26 @@
       </c>
     </row>
     <row r="2" spans="2:49" x14ac:dyDescent="0.25">
-      <c r="Z2" s="193" t="s">
+      <c r="Z2" s="149" t="s">
         <v>269</v>
       </c>
-      <c r="AA2" s="193"/>
-      <c r="AE2" s="193" t="s">
+      <c r="AA2" s="149"/>
+      <c r="AE2" s="149" t="s">
         <v>4</v>
       </c>
-      <c r="AF2" s="193"/>
-      <c r="AK2" s="193" t="s">
+      <c r="AF2" s="149"/>
+      <c r="AK2" s="149" t="s">
         <v>259</v>
       </c>
-      <c r="AL2" s="193"/>
-      <c r="AP2" s="193" t="s">
+      <c r="AL2" s="149"/>
+      <c r="AP2" s="149" t="s">
         <v>258</v>
       </c>
-      <c r="AQ2" s="193"/>
-      <c r="AV2" s="193" t="s">
+      <c r="AQ2" s="149"/>
+      <c r="AV2" s="149" t="s">
         <v>262</v>
       </c>
-      <c r="AW2" s="193"/>
+      <c r="AW2" s="149"/>
     </row>
     <row r="3" spans="2:49" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
@@ -40461,10 +40481,10 @@
       <c r="S3" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="V3" s="193" t="s">
+      <c r="V3" s="149" t="s">
         <v>245</v>
       </c>
-      <c r="W3" s="193"/>
+      <c r="W3" s="149"/>
       <c r="Z3" s="102" t="s">
         <v>244</v>
       </c>
@@ -40913,10 +40933,19 @@
         <f>+F8-I8-J8-K8-L8-M8</f>
         <v>71556.068299415332</v>
       </c>
-      <c r="O8" s="7"/>
-      <c r="P8" s="7"/>
-      <c r="Q8" s="9"/>
-      <c r="R8" s="2"/>
+      <c r="O8" s="7">
+        <v>71556.070000000007</v>
+      </c>
+      <c r="P8" s="7">
+        <f>+N8-O8</f>
+        <v>-1.7005846748361364E-3</v>
+      </c>
+      <c r="Q8" s="9">
+        <v>46233</v>
+      </c>
+      <c r="R8" s="2">
+        <v>18</v>
+      </c>
       <c r="S8" s="12">
         <v>124</v>
       </c>
@@ -40979,7 +41008,7 @@
       </c>
       <c r="O10" s="20">
         <f t="shared" si="4"/>
-        <v>97734.111442501075</v>
+        <v>169290.18144250108</v>
       </c>
       <c r="Q10" s="74"/>
       <c r="V10" s="105" t="s">
@@ -41091,22 +41120,22 @@
       </c>
     </row>
     <row r="2" spans="2:42" x14ac:dyDescent="0.25">
-      <c r="Z2" s="193" t="s">
+      <c r="Z2" s="149" t="s">
         <v>269</v>
       </c>
-      <c r="AA2" s="193"/>
-      <c r="AE2" s="193" t="s">
+      <c r="AA2" s="149"/>
+      <c r="AE2" s="149" t="s">
         <v>259</v>
       </c>
-      <c r="AF2" s="193"/>
-      <c r="AJ2" s="193" t="s">
+      <c r="AF2" s="149"/>
+      <c r="AJ2" s="149" t="s">
         <v>258</v>
       </c>
-      <c r="AK2" s="193"/>
-      <c r="AO2" s="193" t="s">
+      <c r="AK2" s="149"/>
+      <c r="AO2" s="149" t="s">
         <v>262</v>
       </c>
-      <c r="AP2" s="193"/>
+      <c r="AP2" s="149"/>
     </row>
     <row r="3" spans="2:42" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
@@ -41163,10 +41192,10 @@
       <c r="S3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="V3" s="193" t="s">
+      <c r="V3" s="149" t="s">
         <v>245</v>
       </c>
-      <c r="W3" s="193"/>
+      <c r="W3" s="149"/>
       <c r="Z3" s="102" t="s">
         <v>244</v>
       </c>
@@ -41514,9 +41543,16 @@
         <f>+F7-I7-J7-K7-L7-M7</f>
         <v>2565.1499999999996</v>
       </c>
-      <c r="O7" s="7"/>
-      <c r="P7" s="7"/>
-      <c r="Q7" s="9"/>
+      <c r="O7" s="7">
+        <v>2565.15</v>
+      </c>
+      <c r="P7" s="7">
+        <f>+N7-O7</f>
+        <v>0</v>
+      </c>
+      <c r="Q7" s="9">
+        <v>46233</v>
+      </c>
       <c r="R7" s="12">
         <v>125</v>
       </c>
@@ -41579,7 +41615,7 @@
       </c>
       <c r="O9" s="20">
         <f t="shared" si="0"/>
-        <v>89121.463749999995</v>
+        <v>91686.61374999999</v>
       </c>
     </row>
     <row r="11" spans="2:42" x14ac:dyDescent="0.25">
@@ -41644,67 +41680,67 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B2" s="203" t="s">
+      <c r="B2" s="191" t="s">
         <v>59</v>
       </c>
-      <c r="C2" s="202" t="s">
+      <c r="C2" s="190" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="202" t="s">
+      <c r="D2" s="190" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="205" t="s">
+      <c r="E2" s="193" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="202" t="s">
+      <c r="F2" s="190" t="s">
         <v>43</v>
       </c>
-      <c r="G2" s="202"/>
-      <c r="H2" s="202"/>
-      <c r="I2" s="161" t="s">
+      <c r="G2" s="190"/>
+      <c r="H2" s="190"/>
+      <c r="I2" s="150" t="s">
         <v>44</v>
       </c>
-      <c r="J2" s="196"/>
-      <c r="K2" s="196"/>
-      <c r="L2" s="196"/>
-      <c r="M2" s="162"/>
-      <c r="N2" s="212" t="s">
+      <c r="J2" s="184"/>
+      <c r="K2" s="184"/>
+      <c r="L2" s="184"/>
+      <c r="M2" s="151"/>
+      <c r="N2" s="201" t="s">
         <v>7</v>
       </c>
-      <c r="O2" s="212" t="s">
+      <c r="O2" s="201" t="s">
         <v>8</v>
       </c>
-      <c r="P2" s="213" t="s">
+      <c r="P2" s="202" t="s">
         <v>15</v>
       </c>
-      <c r="Q2" s="202" t="s">
+      <c r="Q2" s="190" t="s">
         <v>17</v>
       </c>
-      <c r="R2" s="202" t="s">
+      <c r="R2" s="190" t="s">
         <v>18</v>
       </c>
-      <c r="U2" s="150" t="s">
+      <c r="U2" s="198" t="s">
         <v>245</v>
       </c>
-      <c r="V2" s="150"/>
-      <c r="AA2" s="207" t="s">
+      <c r="V2" s="198"/>
+      <c r="AA2" s="195" t="s">
         <v>300</v>
       </c>
-      <c r="AB2" s="207"/>
-      <c r="AC2" s="207"/>
-      <c r="AD2" s="207"/>
-      <c r="AE2" s="207"/>
-      <c r="AF2" s="207"/>
-      <c r="AH2" s="207" t="s">
+      <c r="AB2" s="195"/>
+      <c r="AC2" s="195"/>
+      <c r="AD2" s="195"/>
+      <c r="AE2" s="195"/>
+      <c r="AF2" s="195"/>
+      <c r="AH2" s="195" t="s">
         <v>301</v>
       </c>
-      <c r="AI2" s="207"/>
+      <c r="AI2" s="195"/>
     </row>
     <row r="3" spans="2:35" x14ac:dyDescent="0.25">
-      <c r="B3" s="204"/>
-      <c r="C3" s="202"/>
-      <c r="D3" s="202"/>
-      <c r="E3" s="206"/>
+      <c r="B3" s="192"/>
+      <c r="C3" s="190"/>
+      <c r="D3" s="190"/>
+      <c r="E3" s="194"/>
       <c r="F3" s="21" t="s">
         <v>3</v>
       </c>
@@ -41723,15 +41759,15 @@
       <c r="K3" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="L3" s="197" t="s">
+      <c r="L3" s="185" t="s">
         <v>6</v>
       </c>
-      <c r="M3" s="198"/>
-      <c r="N3" s="212"/>
-      <c r="O3" s="212"/>
-      <c r="P3" s="214"/>
-      <c r="Q3" s="202"/>
-      <c r="R3" s="202"/>
+      <c r="M3" s="186"/>
+      <c r="N3" s="201"/>
+      <c r="O3" s="201"/>
+      <c r="P3" s="203"/>
+      <c r="Q3" s="190"/>
+      <c r="R3" s="190"/>
       <c r="U3" s="7" t="s">
         <v>251</v>
       </c>
@@ -41768,7 +41804,7 @@
       <c r="B4" s="24">
         <v>2</v>
       </c>
-      <c r="C4" s="194">
+      <c r="C4" s="182">
         <v>45809</v>
       </c>
       <c r="D4" s="2" t="s">
@@ -41803,7 +41839,7 @@
         <f>+F4*I4-K4</f>
         <v>87560.986819576647</v>
       </c>
-      <c r="M4" s="199">
+      <c r="M4" s="187">
         <f>+L4+L5</f>
         <v>560177.05703168991</v>
       </c>
@@ -41820,7 +41856,7 @@
       <c r="Q4" s="2">
         <v>6</v>
       </c>
-      <c r="R4" s="208" t="s">
+      <c r="R4" s="196" t="s">
         <v>49</v>
       </c>
       <c r="U4" s="7" t="s">
@@ -41856,7 +41892,7 @@
       <c r="B5" s="72">
         <v>3</v>
       </c>
-      <c r="C5" s="195"/>
+      <c r="C5" s="183"/>
       <c r="D5" s="91" t="s">
         <v>42</v>
       </c>
@@ -41889,7 +41925,7 @@
         <f>+F5*I5-K5</f>
         <v>472616.07021211332</v>
       </c>
-      <c r="M5" s="200"/>
+      <c r="M5" s="188"/>
       <c r="N5" s="93">
         <v>472616.07</v>
       </c>
@@ -41903,7 +41939,7 @@
       <c r="Q5" s="91">
         <v>6</v>
       </c>
-      <c r="R5" s="209"/>
+      <c r="R5" s="197"/>
       <c r="U5" s="7" t="s">
         <v>252</v>
       </c>
@@ -42022,7 +42058,7 @@
       <c r="B7" s="12">
         <v>6</v>
       </c>
-      <c r="C7" s="194">
+      <c r="C7" s="182">
         <v>46143</v>
       </c>
       <c r="D7" s="2" t="s">
@@ -42057,25 +42093,25 @@
         <f>+F7*I7-K7</f>
         <v>-525022.25</v>
       </c>
-      <c r="M7" s="201">
+      <c r="M7" s="189">
         <f>+L7+L8</f>
         <v>-421910.2</v>
       </c>
-      <c r="N7" s="201">
+      <c r="N7" s="189">
         <f>+M7</f>
         <v>-421910.2</v>
       </c>
-      <c r="O7" s="201">
+      <c r="O7" s="189">
         <f>+M7-N7</f>
         <v>0</v>
       </c>
-      <c r="P7" s="210">
+      <c r="P7" s="199">
         <v>46198</v>
       </c>
       <c r="Q7" s="2">
         <v>17</v>
       </c>
-      <c r="R7" s="207" t="s">
+      <c r="R7" s="195" t="s">
         <v>232</v>
       </c>
       <c r="U7" s="7" t="s">
@@ -42090,7 +42126,7 @@
       <c r="B8" s="12">
         <v>13</v>
       </c>
-      <c r="C8" s="195"/>
+      <c r="C8" s="183"/>
       <c r="D8" s="2" t="s">
         <v>225</v>
       </c>
@@ -42123,14 +42159,14 @@
         <f>+F8*I8-K8</f>
         <v>103112.04999999999</v>
       </c>
-      <c r="M8" s="201"/>
-      <c r="N8" s="201"/>
-      <c r="O8" s="201"/>
-      <c r="P8" s="211"/>
+      <c r="M8" s="189"/>
+      <c r="N8" s="189"/>
+      <c r="O8" s="189"/>
+      <c r="P8" s="200"/>
       <c r="Q8" s="2">
         <v>17</v>
       </c>
-      <c r="R8" s="207"/>
+      <c r="R8" s="195"/>
     </row>
     <row r="9" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B9" s="13"/>
@@ -42322,50 +42358,50 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B2" s="202" t="s">
+      <c r="B2" s="190" t="s">
         <v>59</v>
       </c>
-      <c r="C2" s="202" t="s">
+      <c r="C2" s="190" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="202" t="s">
+      <c r="D2" s="190" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="202" t="s">
+      <c r="E2" s="190" t="s">
         <v>43</v>
       </c>
-      <c r="F2" s="202"/>
-      <c r="G2" s="202"/>
-      <c r="H2" s="161" t="s">
+      <c r="F2" s="190"/>
+      <c r="G2" s="190"/>
+      <c r="H2" s="150" t="s">
         <v>44</v>
       </c>
-      <c r="I2" s="196"/>
-      <c r="J2" s="196"/>
-      <c r="K2" s="196"/>
-      <c r="L2" s="162"/>
-      <c r="M2" s="212" t="s">
+      <c r="I2" s="184"/>
+      <c r="J2" s="184"/>
+      <c r="K2" s="184"/>
+      <c r="L2" s="151"/>
+      <c r="M2" s="201" t="s">
         <v>7</v>
       </c>
-      <c r="N2" s="212" t="s">
+      <c r="N2" s="201" t="s">
         <v>8</v>
       </c>
-      <c r="O2" s="213" t="s">
+      <c r="O2" s="202" t="s">
         <v>15</v>
       </c>
-      <c r="P2" s="202" t="s">
+      <c r="P2" s="190" t="s">
         <v>17</v>
       </c>
-      <c r="Q2" s="202" t="s">
+      <c r="Q2" s="190" t="s">
         <v>18</v>
       </c>
-      <c r="R2" s="202" t="s">
+      <c r="R2" s="190" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="3" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B3" s="202"/>
-      <c r="C3" s="202"/>
-      <c r="D3" s="202"/>
+      <c r="B3" s="190"/>
+      <c r="C3" s="190"/>
+      <c r="D3" s="190"/>
       <c r="E3" s="21" t="s">
         <v>3</v>
       </c>
@@ -42384,38 +42420,38 @@
       <c r="J3" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="K3" s="197" t="s">
+      <c r="K3" s="185" t="s">
         <v>6</v>
       </c>
-      <c r="L3" s="198"/>
-      <c r="M3" s="212"/>
-      <c r="N3" s="212"/>
-      <c r="O3" s="214"/>
-      <c r="P3" s="202"/>
-      <c r="Q3" s="202"/>
-      <c r="R3" s="202"/>
-      <c r="U3" s="150" t="s">
+      <c r="L3" s="186"/>
+      <c r="M3" s="201"/>
+      <c r="N3" s="201"/>
+      <c r="O3" s="203"/>
+      <c r="P3" s="190"/>
+      <c r="Q3" s="190"/>
+      <c r="R3" s="190"/>
+      <c r="U3" s="198" t="s">
         <v>245</v>
       </c>
-      <c r="V3" s="150"/>
-      <c r="Y3" s="207" t="s">
+      <c r="V3" s="198"/>
+      <c r="Y3" s="195" t="s">
         <v>304</v>
       </c>
-      <c r="Z3" s="207"/>
-      <c r="AA3" s="207"/>
-      <c r="AC3" s="207" t="s">
+      <c r="Z3" s="195"/>
+      <c r="AA3" s="195"/>
+      <c r="AC3" s="195" t="s">
         <v>301</v>
       </c>
-      <c r="AD3" s="207"/>
+      <c r="AD3" s="195"/>
     </row>
     <row r="4" spans="2:30" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="177">
+      <c r="B4" s="166">
         <v>5</v>
       </c>
-      <c r="C4" s="222">
+      <c r="C4" s="211">
         <v>46082</v>
       </c>
-      <c r="D4" s="177" t="s">
+      <c r="D4" s="166" t="s">
         <v>185</v>
       </c>
       <c r="E4" s="7">
@@ -42444,22 +42480,22 @@
         <f>+E4*H4-J4</f>
         <v>84326.527793167479</v>
       </c>
-      <c r="L4" s="199">
+      <c r="L4" s="187">
         <f>+K4+K5</f>
         <v>84853.966913182536</v>
       </c>
-      <c r="M4" s="215">
+      <c r="M4" s="204">
         <f>+K4+K5</f>
         <v>84853.966913182536</v>
       </c>
-      <c r="N4" s="215">
+      <c r="N4" s="204">
         <f>+K4+K5-M4</f>
         <v>0</v>
       </c>
-      <c r="O4" s="191">
+      <c r="O4" s="180">
         <v>46141</v>
       </c>
-      <c r="P4" s="177">
+      <c r="P4" s="166">
         <v>15</v>
       </c>
       <c r="Q4" s="12">
@@ -42492,9 +42528,9 @@
       </c>
     </row>
     <row r="5" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B5" s="177"/>
-      <c r="C5" s="222"/>
-      <c r="D5" s="177"/>
+      <c r="B5" s="166"/>
+      <c r="C5" s="211"/>
+      <c r="D5" s="166"/>
       <c r="E5" s="7">
         <v>6693.3096551176686</v>
       </c>
@@ -42521,11 +42557,11 @@
         <f>+E5*H5-J5</f>
         <v>527.43912001505078</v>
       </c>
-      <c r="L5" s="221"/>
-      <c r="M5" s="177"/>
-      <c r="N5" s="177"/>
-      <c r="O5" s="177"/>
-      <c r="P5" s="177"/>
+      <c r="L5" s="210"/>
+      <c r="M5" s="166"/>
+      <c r="N5" s="166"/>
+      <c r="O5" s="166"/>
+      <c r="P5" s="166"/>
       <c r="Q5" s="12">
         <v>109</v>
       </c>
@@ -42559,13 +42595,13 @@
       </c>
     </row>
     <row r="6" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B6" s="177">
+      <c r="B6" s="166">
         <v>5</v>
       </c>
-      <c r="C6" s="194">
+      <c r="C6" s="182">
         <v>46113</v>
       </c>
-      <c r="D6" s="220" t="s">
+      <c r="D6" s="209" t="s">
         <v>210</v>
       </c>
       <c r="E6" s="81">
@@ -42594,28 +42630,28 @@
         <f>+E6*H6-J6</f>
         <v>1340.2285312500001</v>
       </c>
-      <c r="L6" s="199">
+      <c r="L6" s="187">
         <f>+K6+K7</f>
         <v>2049.2173564683389</v>
       </c>
-      <c r="M6" s="215">
+      <c r="M6" s="204">
         <f>+K6+K7</f>
         <v>2049.2173564683389</v>
       </c>
-      <c r="N6" s="215">
+      <c r="N6" s="204">
         <f>+K6+K7-M6</f>
         <v>0</v>
       </c>
-      <c r="O6" s="216">
+      <c r="O6" s="205">
         <v>46163</v>
       </c>
-      <c r="P6" s="177">
+      <c r="P6" s="166">
         <v>16</v>
       </c>
-      <c r="Q6" s="177">
+      <c r="Q6" s="166">
         <v>113</v>
       </c>
-      <c r="R6" s="218" t="s">
+      <c r="R6" s="207" t="s">
         <v>213</v>
       </c>
       <c r="U6" s="7" t="s">
@@ -42645,9 +42681,9 @@
       </c>
     </row>
     <row r="7" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B7" s="177"/>
-      <c r="C7" s="195"/>
-      <c r="D7" s="217"/>
+      <c r="B7" s="166"/>
+      <c r="C7" s="183"/>
+      <c r="D7" s="206"/>
       <c r="E7" s="81">
         <v>6693.3096551176686</v>
       </c>
@@ -42674,13 +42710,13 @@
         <f>+E7*H7-J7</f>
         <v>708.98882521833912</v>
       </c>
-      <c r="L7" s="221"/>
-      <c r="M7" s="177"/>
-      <c r="N7" s="177"/>
-      <c r="O7" s="217"/>
-      <c r="P7" s="177"/>
-      <c r="Q7" s="177"/>
-      <c r="R7" s="219"/>
+      <c r="L7" s="210"/>
+      <c r="M7" s="166"/>
+      <c r="N7" s="166"/>
+      <c r="O7" s="206"/>
+      <c r="P7" s="166"/>
+      <c r="Q7" s="166"/>
+      <c r="R7" s="208"/>
       <c r="U7" s="7" t="s">
         <v>247</v>
       </c>
@@ -42708,13 +42744,13 @@
       </c>
     </row>
     <row r="8" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B8" s="177">
+      <c r="B8" s="166">
         <v>5</v>
       </c>
-      <c r="C8" s="194">
+      <c r="C8" s="182">
         <v>46143</v>
       </c>
-      <c r="D8" s="220" t="s">
+      <c r="D8" s="209" t="s">
         <v>228</v>
       </c>
       <c r="E8" s="81">
@@ -42743,28 +42779,28 @@
         <f t="shared" ref="K8:K11" si="5">+E8*H8-J8</f>
         <v>9265.7774999999983</v>
       </c>
-      <c r="L8" s="199">
+      <c r="L8" s="187">
         <f>+K8+K9</f>
         <v>9857.7021126977561</v>
       </c>
-      <c r="M8" s="215">
+      <c r="M8" s="204">
         <f>+L8</f>
         <v>9857.7021126977561</v>
       </c>
-      <c r="N8" s="215">
+      <c r="N8" s="204">
         <f>+K8+K9-M8</f>
         <v>0</v>
       </c>
-      <c r="O8" s="216">
+      <c r="O8" s="205">
         <v>46198</v>
       </c>
-      <c r="P8" s="177">
+      <c r="P8" s="166">
         <v>17</v>
       </c>
-      <c r="Q8" s="177">
+      <c r="Q8" s="166">
         <v>119</v>
       </c>
-      <c r="R8" s="218" t="s">
+      <c r="R8" s="207" t="s">
         <v>231</v>
       </c>
       <c r="U8" s="7" t="s">
@@ -42772,14 +42808,14 @@
       </c>
       <c r="V8" s="7">
         <f>+M13</f>
-        <v>96760.886382348632</v>
+        <v>98809.886382348632</v>
       </c>
       <c r="Z8" s="8"/>
     </row>
     <row r="9" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B9" s="177"/>
-      <c r="C9" s="195"/>
-      <c r="D9" s="217"/>
+      <c r="B9" s="166"/>
+      <c r="C9" s="183"/>
+      <c r="D9" s="206"/>
       <c r="E9" s="81">
         <v>6693.3096551176686</v>
       </c>
@@ -42806,22 +42842,22 @@
         <f t="shared" si="5"/>
         <v>591.92461269775856</v>
       </c>
-      <c r="L9" s="221"/>
-      <c r="M9" s="177"/>
-      <c r="N9" s="177"/>
-      <c r="O9" s="217"/>
-      <c r="P9" s="177"/>
-      <c r="Q9" s="177"/>
-      <c r="R9" s="219"/>
+      <c r="L9" s="210"/>
+      <c r="M9" s="166"/>
+      <c r="N9" s="166"/>
+      <c r="O9" s="206"/>
+      <c r="P9" s="166"/>
+      <c r="Q9" s="166"/>
+      <c r="R9" s="208"/>
     </row>
     <row r="10" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B10" s="177">
+      <c r="B10" s="166">
         <v>5</v>
       </c>
-      <c r="C10" s="194">
+      <c r="C10" s="182">
         <v>46174</v>
       </c>
-      <c r="D10" s="220" t="s">
+      <c r="D10" s="209" t="s">
         <v>313</v>
       </c>
       <c r="E10" s="81">
@@ -42850,20 +42886,33 @@
         <f t="shared" si="5"/>
         <v>1340.2285312500001</v>
       </c>
-      <c r="L10" s="199"/>
-      <c r="M10" s="215"/>
-      <c r="N10" s="215"/>
-      <c r="O10" s="216"/>
-      <c r="P10" s="177"/>
-      <c r="Q10" s="177"/>
-      <c r="R10" s="218" t="s">
+      <c r="L10" s="187">
+        <v>2049</v>
+      </c>
+      <c r="M10" s="204">
+        <v>2049</v>
+      </c>
+      <c r="N10" s="204">
+        <f>+K10+K11-M10</f>
+        <v>0.21735646833894862</v>
+      </c>
+      <c r="O10" s="205">
+        <v>46233</v>
+      </c>
+      <c r="P10" s="166">
+        <v>18</v>
+      </c>
+      <c r="Q10" s="166">
+        <v>126</v>
+      </c>
+      <c r="R10" s="207" t="s">
         <v>312</v>
       </c>
     </row>
     <row r="11" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B11" s="177"/>
-      <c r="C11" s="195"/>
-      <c r="D11" s="217"/>
+      <c r="B11" s="166"/>
+      <c r="C11" s="183"/>
+      <c r="D11" s="206"/>
       <c r="E11" s="81">
         <v>6693.3096551176686</v>
       </c>
@@ -42890,13 +42939,13 @@
         <f t="shared" si="5"/>
         <v>708.98882521833912</v>
       </c>
-      <c r="L11" s="221"/>
-      <c r="M11" s="177"/>
-      <c r="N11" s="177"/>
-      <c r="O11" s="217"/>
-      <c r="P11" s="177"/>
-      <c r="Q11" s="177"/>
-      <c r="R11" s="219"/>
+      <c r="L11" s="210"/>
+      <c r="M11" s="166"/>
+      <c r="N11" s="166"/>
+      <c r="O11" s="206"/>
+      <c r="P11" s="166"/>
+      <c r="Q11" s="166"/>
+      <c r="R11" s="208"/>
     </row>
     <row r="12" spans="2:30" x14ac:dyDescent="0.25">
       <c r="B12" s="13"/>
@@ -42926,7 +42975,7 @@
       <c r="L13" s="22"/>
       <c r="M13" s="22">
         <f>SUM(M4:M11)</f>
-        <v>96760.886382348632</v>
+        <v>98809.886382348632</v>
       </c>
     </row>
   </sheetData>
@@ -43016,47 +43065,47 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B2" s="202" t="s">
+      <c r="B2" s="190" t="s">
         <v>59</v>
       </c>
-      <c r="C2" s="202" t="s">
+      <c r="C2" s="190" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="202" t="s">
+      <c r="D2" s="190" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="202" t="s">
+      <c r="E2" s="190" t="s">
         <v>43</v>
       </c>
-      <c r="F2" s="202"/>
-      <c r="G2" s="202"/>
-      <c r="H2" s="161" t="s">
+      <c r="F2" s="190"/>
+      <c r="G2" s="190"/>
+      <c r="H2" s="150" t="s">
         <v>44</v>
       </c>
-      <c r="I2" s="196"/>
-      <c r="J2" s="196"/>
-      <c r="K2" s="196"/>
-      <c r="L2" s="162"/>
-      <c r="M2" s="212" t="s">
+      <c r="I2" s="184"/>
+      <c r="J2" s="184"/>
+      <c r="K2" s="184"/>
+      <c r="L2" s="151"/>
+      <c r="M2" s="201" t="s">
         <v>7</v>
       </c>
-      <c r="N2" s="212" t="s">
+      <c r="N2" s="201" t="s">
         <v>8</v>
       </c>
-      <c r="O2" s="213" t="s">
+      <c r="O2" s="202" t="s">
         <v>15</v>
       </c>
-      <c r="P2" s="202" t="s">
+      <c r="P2" s="190" t="s">
         <v>18</v>
       </c>
-      <c r="Q2" s="202" t="s">
+      <c r="Q2" s="190" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="3" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B3" s="202"/>
-      <c r="C3" s="202"/>
-      <c r="D3" s="202"/>
+      <c r="B3" s="190"/>
+      <c r="C3" s="190"/>
+      <c r="D3" s="190"/>
       <c r="E3" s="21" t="s">
         <v>3</v>
       </c>
@@ -43075,37 +43124,37 @@
       <c r="J3" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="K3" s="197" t="s">
+      <c r="K3" s="185" t="s">
         <v>6</v>
       </c>
-      <c r="L3" s="198"/>
-      <c r="M3" s="212"/>
-      <c r="N3" s="212"/>
-      <c r="O3" s="214"/>
-      <c r="P3" s="202"/>
-      <c r="Q3" s="202"/>
-      <c r="T3" s="150" t="s">
+      <c r="L3" s="186"/>
+      <c r="M3" s="201"/>
+      <c r="N3" s="201"/>
+      <c r="O3" s="203"/>
+      <c r="P3" s="190"/>
+      <c r="Q3" s="190"/>
+      <c r="T3" s="198" t="s">
         <v>245</v>
       </c>
-      <c r="U3" s="150"/>
-      <c r="Y3" s="207" t="s">
+      <c r="U3" s="198"/>
+      <c r="Y3" s="195" t="s">
         <v>304</v>
       </c>
-      <c r="Z3" s="207"/>
-      <c r="AA3" s="207"/>
-      <c r="AC3" s="207" t="s">
+      <c r="Z3" s="195"/>
+      <c r="AA3" s="195"/>
+      <c r="AC3" s="195" t="s">
         <v>301</v>
       </c>
-      <c r="AD3" s="207"/>
+      <c r="AD3" s="195"/>
     </row>
     <row r="4" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B4" s="220">
+      <c r="B4" s="209">
         <v>5</v>
       </c>
-      <c r="C4" s="194">
+      <c r="C4" s="182">
         <v>46082</v>
       </c>
-      <c r="D4" s="220" t="s">
+      <c r="D4" s="209" t="s">
         <v>189</v>
       </c>
       <c r="E4" s="7">
@@ -43133,19 +43182,19 @@
         <f t="shared" ref="K4:K11" si="2">+E4*H4-J4</f>
         <v>-84326.527793167479</v>
       </c>
-      <c r="L4" s="199">
+      <c r="L4" s="187">
         <f>+K4+K5</f>
         <v>-84853.966913182536</v>
       </c>
-      <c r="M4" s="215">
+      <c r="M4" s="204">
         <f>+K4+K5</f>
         <v>-84853.966913182536</v>
       </c>
-      <c r="N4" s="215">
+      <c r="N4" s="204">
         <f>+K4+K5-M4</f>
         <v>0</v>
       </c>
-      <c r="O4" s="191">
+      <c r="O4" s="180">
         <v>46141</v>
       </c>
       <c r="P4" s="2" t="s">
@@ -43178,9 +43227,9 @@
       </c>
     </row>
     <row r="5" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B5" s="217"/>
-      <c r="C5" s="195"/>
-      <c r="D5" s="217"/>
+      <c r="B5" s="206"/>
+      <c r="C5" s="183"/>
+      <c r="D5" s="206"/>
       <c r="E5" s="7">
         <v>-6693.3096551176686</v>
       </c>
@@ -43206,10 +43255,10 @@
         <f t="shared" si="2"/>
         <v>-527.43912001505078</v>
       </c>
-      <c r="L5" s="221"/>
-      <c r="M5" s="177"/>
-      <c r="N5" s="177"/>
-      <c r="O5" s="177"/>
+      <c r="L5" s="210"/>
+      <c r="M5" s="166"/>
+      <c r="N5" s="166"/>
+      <c r="O5" s="166"/>
       <c r="P5" s="2" t="s">
         <v>187</v>
       </c>
@@ -43243,13 +43292,13 @@
       </c>
     </row>
     <row r="6" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B6" s="220">
+      <c r="B6" s="209">
         <v>5</v>
       </c>
-      <c r="C6" s="194">
+      <c r="C6" s="182">
         <v>46113</v>
       </c>
-      <c r="D6" s="220" t="s">
+      <c r="D6" s="209" t="s">
         <v>214</v>
       </c>
       <c r="E6" s="81">
@@ -43277,25 +43326,25 @@
         <f t="shared" si="2"/>
         <v>-1340.2285312500001</v>
       </c>
-      <c r="L6" s="199">
+      <c r="L6" s="187">
         <f>+K6+K7</f>
         <v>-2049.2173564683394</v>
       </c>
-      <c r="M6" s="215">
+      <c r="M6" s="204">
         <f>+K6+K7</f>
         <v>-2049.2173564683394</v>
       </c>
-      <c r="N6" s="215">
+      <c r="N6" s="204">
         <f>+K6+K7-M6</f>
         <v>0</v>
       </c>
-      <c r="O6" s="191">
+      <c r="O6" s="180">
         <v>46163</v>
       </c>
-      <c r="P6" s="168" t="s">
+      <c r="P6" s="157" t="s">
         <v>215</v>
       </c>
-      <c r="Q6" s="218" t="s">
+      <c r="Q6" s="207" t="s">
         <v>213</v>
       </c>
       <c r="T6" s="7" t="s">
@@ -43325,9 +43374,9 @@
       </c>
     </row>
     <row r="7" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B7" s="217"/>
-      <c r="C7" s="195"/>
-      <c r="D7" s="217"/>
+      <c r="B7" s="206"/>
+      <c r="C7" s="183"/>
+      <c r="D7" s="206"/>
       <c r="E7" s="81">
         <v>-6693.3096551176704</v>
       </c>
@@ -43353,12 +43402,12 @@
         <f t="shared" si="2"/>
         <v>-708.98882521833923</v>
       </c>
-      <c r="L7" s="221"/>
-      <c r="M7" s="177"/>
-      <c r="N7" s="177"/>
-      <c r="O7" s="177"/>
-      <c r="P7" s="168"/>
-      <c r="Q7" s="219"/>
+      <c r="L7" s="210"/>
+      <c r="M7" s="166"/>
+      <c r="N7" s="166"/>
+      <c r="O7" s="166"/>
+      <c r="P7" s="157"/>
+      <c r="Q7" s="208"/>
       <c r="T7" s="7" t="s">
         <v>247</v>
       </c>
@@ -43386,13 +43435,13 @@
       </c>
     </row>
     <row r="8" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B8" s="220">
+      <c r="B8" s="209">
         <v>5</v>
       </c>
-      <c r="C8" s="194">
+      <c r="C8" s="182">
         <v>46143</v>
       </c>
-      <c r="D8" s="220" t="s">
+      <c r="D8" s="209" t="s">
         <v>229</v>
       </c>
       <c r="E8" s="81">
@@ -43420,25 +43469,25 @@
         <f t="shared" si="2"/>
         <v>-9265.7774999999983</v>
       </c>
-      <c r="L8" s="199">
+      <c r="L8" s="187">
         <f>+K8+K9</f>
         <v>-9857.7021126977561</v>
       </c>
-      <c r="M8" s="215">
+      <c r="M8" s="204">
         <f>+L8</f>
         <v>-9857.7021126977561</v>
       </c>
-      <c r="N8" s="215">
+      <c r="N8" s="204">
         <f>+K8+K9-M8</f>
         <v>0</v>
       </c>
-      <c r="O8" s="191">
+      <c r="O8" s="180">
         <v>46198</v>
       </c>
-      <c r="P8" s="168" t="s">
+      <c r="P8" s="157" t="s">
         <v>230</v>
       </c>
-      <c r="Q8" s="218" t="s">
+      <c r="Q8" s="207" t="s">
         <v>231</v>
       </c>
       <c r="T8" s="7" t="s">
@@ -43446,13 +43495,13 @@
       </c>
       <c r="U8" s="7">
         <f>+M13</f>
-        <v>-96760.886382348632</v>
+        <v>-98809.886382348632</v>
       </c>
     </row>
     <row r="9" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B9" s="217"/>
-      <c r="C9" s="195"/>
-      <c r="D9" s="217"/>
+      <c r="B9" s="206"/>
+      <c r="C9" s="183"/>
+      <c r="D9" s="206"/>
       <c r="E9" s="81">
         <v>-6693.3096551176704</v>
       </c>
@@ -43478,21 +43527,21 @@
         <f t="shared" si="2"/>
         <v>-591.92461269775868</v>
       </c>
-      <c r="L9" s="221"/>
-      <c r="M9" s="177"/>
-      <c r="N9" s="177"/>
-      <c r="O9" s="177"/>
-      <c r="P9" s="168"/>
-      <c r="Q9" s="219"/>
+      <c r="L9" s="210"/>
+      <c r="M9" s="166"/>
+      <c r="N9" s="166"/>
+      <c r="O9" s="166"/>
+      <c r="P9" s="157"/>
+      <c r="Q9" s="208"/>
     </row>
     <row r="10" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B10" s="177">
+      <c r="B10" s="166">
         <v>5</v>
       </c>
-      <c r="C10" s="194">
+      <c r="C10" s="182">
         <v>46174</v>
       </c>
-      <c r="D10" s="220" t="s">
+      <c r="D10" s="209" t="s">
         <v>314</v>
       </c>
       <c r="E10" s="81">
@@ -43521,22 +43570,31 @@
         <f t="shared" si="2"/>
         <v>-1340.2285312500001</v>
       </c>
-      <c r="L10" s="199">
+      <c r="L10" s="187">
         <f>+K10+K11</f>
         <v>-2049.2173564683394</v>
       </c>
-      <c r="M10" s="215"/>
-      <c r="N10" s="215"/>
-      <c r="O10" s="216"/>
-      <c r="P10" s="177"/>
-      <c r="Q10" s="218" t="s">
+      <c r="M10" s="204">
+        <v>-2049</v>
+      </c>
+      <c r="N10" s="204">
+        <f>+K10+K11-M10</f>
+        <v>-0.21735646833940336</v>
+      </c>
+      <c r="O10" s="205">
+        <v>46233</v>
+      </c>
+      <c r="P10" s="157" t="s">
+        <v>325</v>
+      </c>
+      <c r="Q10" s="207" t="s">
         <v>312</v>
       </c>
     </row>
     <row r="11" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B11" s="177"/>
-      <c r="C11" s="195"/>
-      <c r="D11" s="217"/>
+      <c r="B11" s="166"/>
+      <c r="C11" s="183"/>
+      <c r="D11" s="206"/>
       <c r="E11" s="81">
         <v>-6693.3096551176704</v>
       </c>
@@ -43563,12 +43621,12 @@
         <f t="shared" si="2"/>
         <v>-708.98882521833923</v>
       </c>
-      <c r="L11" s="221"/>
-      <c r="M11" s="177"/>
-      <c r="N11" s="177"/>
-      <c r="O11" s="217"/>
-      <c r="P11" s="177"/>
-      <c r="Q11" s="219"/>
+      <c r="L11" s="210"/>
+      <c r="M11" s="166"/>
+      <c r="N11" s="166"/>
+      <c r="O11" s="206"/>
+      <c r="P11" s="157"/>
+      <c r="Q11" s="208"/>
     </row>
     <row r="12" spans="2:30" x14ac:dyDescent="0.25">
       <c r="B12" s="13"/>
@@ -43598,7 +43656,7 @@
       <c r="L13" s="22"/>
       <c r="M13" s="22">
         <f>SUM(M4:M11)</f>
-        <v>-96760.886382348632</v>
+        <v>-98809.886382348632</v>
       </c>
     </row>
   </sheetData>
@@ -43756,10 +43814,10 @@
       <c r="U2" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="Y2" s="150" t="s">
+      <c r="Y2" s="198" t="s">
         <v>245</v>
       </c>
-      <c r="Z2" s="150"/>
+      <c r="Z2" s="198"/>
       <c r="AL2" s="106" t="str">
         <f t="shared" ref="AL2:AL7" si="0">+C2</f>
         <v>Mes certificado</v>
@@ -44323,7 +44381,7 @@
       </c>
       <c r="Z9" s="7">
         <f>+N24</f>
-        <v>11981219.968249997</v>
+        <v>12964394.143249998</v>
       </c>
       <c r="AL9" s="5">
         <f t="shared" si="10"/>
@@ -44369,7 +44427,7 @@
       <c r="K10" s="7"/>
       <c r="L10" s="7"/>
       <c r="M10" s="7">
-        <f t="shared" ref="M10:M22" si="16">+F10-I10-J10-L10</f>
+        <f t="shared" ref="M10:N22" si="16">+F10-I10-J10-L10</f>
         <v>781003.04849999992</v>
       </c>
       <c r="N10" s="7">
@@ -44822,15 +44880,15 @@
       <c r="Q16" s="2">
         <v>12</v>
       </c>
-      <c r="R16" s="159">
+      <c r="R16" s="220">
         <f>+'Básico $'!F17</f>
         <v>17503240.649999999</v>
       </c>
-      <c r="S16" s="151">
+      <c r="S16" s="212">
         <f>(+F16+F17)/R16</f>
         <v>5.5338895200529627E-2</v>
       </c>
-      <c r="T16" s="151">
+      <c r="T16" s="212">
         <f t="shared" si="17"/>
         <v>-1.3792405489247705E-3</v>
       </c>
@@ -44884,22 +44942,22 @@
         <f t="shared" si="16"/>
         <v>-26503.100000000002</v>
       </c>
-      <c r="N17" s="153">
+      <c r="N17" s="214">
         <f>+M17+M18</f>
         <v>622137.42500000005</v>
       </c>
-      <c r="O17" s="157">
+      <c r="O17" s="218">
         <v>46101</v>
       </c>
-      <c r="P17" s="155" t="s">
+      <c r="P17" s="216" t="s">
         <v>159</v>
       </c>
       <c r="Q17" s="2">
         <v>13</v>
       </c>
-      <c r="R17" s="160"/>
-      <c r="S17" s="152"/>
-      <c r="T17" s="152"/>
+      <c r="R17" s="221"/>
+      <c r="S17" s="213"/>
+      <c r="T17" s="213"/>
       <c r="U17" s="28" t="s">
         <v>150</v>
       </c>
@@ -44950,9 +45008,9 @@
         <f t="shared" si="16"/>
         <v>648640.52500000002</v>
       </c>
-      <c r="N18" s="154"/>
-      <c r="O18" s="158"/>
-      <c r="P18" s="156"/>
+      <c r="N18" s="215"/>
+      <c r="O18" s="219"/>
+      <c r="P18" s="217"/>
       <c r="Q18" s="2">
         <v>14</v>
       </c>
@@ -45220,10 +45278,16 @@
         <f t="shared" si="16"/>
         <v>983174.17499999993</v>
       </c>
-      <c r="N22" s="7"/>
-      <c r="O22" s="9"/>
+      <c r="N22" s="7">
+        <v>983174.17499999993</v>
+      </c>
+      <c r="O22" s="9">
+        <v>46233</v>
+      </c>
       <c r="P22" s="2"/>
-      <c r="Q22" s="2"/>
+      <c r="Q22" s="2">
+        <v>18</v>
+      </c>
       <c r="R22" s="7">
         <f>+'Básico $'!F22</f>
         <v>14976846.560000001</v>
@@ -45292,7 +45356,7 @@
       </c>
       <c r="N24" s="22">
         <f t="shared" si="19"/>
-        <v>11981219.968249997</v>
+        <v>12964394.143249998</v>
       </c>
       <c r="O24" s="29"/>
       <c r="P24" s="29"/>

</xml_diff>